<commit_message>
vault backup: 2026-10-29 12:03:20
</commit_message>
<xml_diff>
--- a/02_Areas/工作经历/鑫犇电子有限公司/01_生产部/工程技术组/设备台账.xlsx
+++ b/02_Areas/工作经历/鑫犇电子有限公司/01_生产部/工程技术组/设备台账.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,8 +74,37 @@
       <i val="1"/>
       <color rgb="004472C4"/>
     </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="001F1F1F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <i val="1"/>
+      <color rgb="002F6475"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00A63D2F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00425066"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -92,8 +121,23 @@
         <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00425066"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCEDEA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -101,11 +145,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D7DFE2"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00425066"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -144,6 +198,27 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -272,94 +347,6 @@
 </comments>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>19050</colOff>
-      <row>0</row>
-      <rowOff>19050</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>495300</colOff>
-      <row>1</row>
-      <rowOff>28575</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Picture 2" descr="eWQHEp"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="0"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData fLocksWithSheet="0" fPrintsWithSheet="1"/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>19050</colOff>
-      <row>0</row>
-      <rowOff>19050</rowOff>
-    </from>
-    <to>
-      <col>0</col>
-      <colOff>1390650</colOff>
-      <row>1</row>
-      <rowOff>247650</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Picture 2" descr="vZPewl"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="0"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData fLocksWithSheet="0" fPrintsWithSheet="1"/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EquipmentRegister" displayName="EquipmentRegister" ref="A1:O9" headerRowCount="1">
   <autoFilter ref="A1:O9"/>
@@ -380,7 +367,7 @@
     <tableColumn id="14" name="备注"/>
     <tableColumn id="15" name="核对状态"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -688,711 +675,711 @@
   <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.466666666666667" defaultRowHeight="18.66666666666666"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" style="6" min="1" max="1"/>
+    <col width="18" customWidth="1" style="6" min="2" max="2"/>
+    <col width="16" customWidth="1" style="6" min="3" max="3"/>
+    <col width="18" customWidth="1" style="6" min="4" max="4"/>
+    <col width="16" customWidth="1" style="6" min="5" max="5"/>
+    <col width="44" customWidth="1" style="6" min="6" max="6"/>
+    <col width="24" customWidth="1" style="6" min="7" max="7"/>
+    <col width="12" customWidth="1" style="6" min="8" max="8"/>
+    <col width="12" customWidth="1" style="6" min="9" max="9"/>
+    <col width="12" customWidth="1" style="6" min="10" max="10"/>
+    <col width="12" customWidth="1" style="6" min="11" max="11"/>
+    <col width="12" customWidth="1" style="6" min="12" max="12"/>
+    <col width="24" customWidth="1" style="6" min="13" max="13"/>
+    <col width="32" customWidth="1" style="6" min="14" max="14"/>
     <col width="16" customWidth="1" style="6" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="37.33333333333333" customHeight="1" s="6">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>设备编号</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>设备名称</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>型号规格</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>品牌/产地</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>类别</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="14" t="inlineStr">
         <is>
           <t>主要技术参数</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="14" t="inlineStr">
         <is>
           <t>工位位置</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="14" t="inlineStr">
         <is>
           <t>责任人</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="14" t="inlineStr">
         <is>
           <t>当前状态</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" s="14" t="inlineStr">
         <is>
           <t>保养等级</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="K1" s="14" t="inlineStr">
         <is>
           <t>上次保养</t>
         </is>
       </c>
-      <c r="L1" s="7" t="inlineStr">
+      <c r="L1" s="14" t="inlineStr">
         <is>
           <t>下次保养</t>
         </is>
       </c>
-      <c r="M1" s="7" t="inlineStr">
+      <c r="M1" s="14" t="inlineStr">
         <is>
           <t>安全防护</t>
         </is>
       </c>
-      <c r="N1" s="7" t="inlineStr">
+      <c r="N1" s="14" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="O1" s="8" t="inlineStr">
+      <c r="O1" s="14" t="inlineStr">
         <is>
           <t>核对状态</t>
         </is>
       </c>
     </row>
     <row r="2" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>SB-001</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>快走丝线切割</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>DK7732</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>泰州四海数控</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>电加工设备</t>
         </is>
       </c>
-      <c r="F2" s="9" t="inlineStr">
+      <c r="F2" s="15" t="inlineStr">
         <is>
           <t>最大加工厚度300mm；锥度±3°；工作台行程320×400mm</t>
         </is>
       </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="G2" s="15" t="inlineStr">
         <is>
           <t>模具车间-线切割区</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" s="16" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I2" s="9" t="inlineStr">
+      <c r="I2" s="15" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J2" s="9" t="inlineStr">
+      <c r="J2" s="15" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K2" s="10" t="inlineStr">
+      <c r="K2" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L2" s="10" t="inlineStr">
+      <c r="L2" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M2" s="9" t="inlineStr">
+      <c r="M2" s="15" t="inlineStr">
         <is>
           <t>防护门/急停已配</t>
         </is>
       </c>
-      <c r="N2" s="11" t="inlineStr">
+      <c r="N2" s="17" t="inlineStr">
         <is>
           <t>双机位油槽，带数控系统</t>
         </is>
       </c>
-      <c r="O2" s="10" t="inlineStr">
+      <c r="O2" s="16" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="3" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>SB-002</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>锥度线切割</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>DK7735</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>电加工设备</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="15" t="inlineStr">
         <is>
           <t>最大加工厚度350mm；大锥度切割；工作台行程350×500mm</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="15" t="inlineStr">
         <is>
           <t>模具车间-线切割区</t>
         </is>
       </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="H3" s="16" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I3" s="9" t="inlineStr">
+      <c r="I3" s="15" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J3" s="9" t="inlineStr">
+      <c r="J3" s="15" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K3" s="10" t="inlineStr">
+      <c r="K3" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L3" s="10" t="inlineStr">
+      <c r="L3" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M3" s="9" t="inlineStr">
+      <c r="M3" s="15" t="inlineStr">
         <is>
           <t>防护门/急停已配</t>
         </is>
       </c>
-      <c r="N3" s="11" t="inlineStr">
+      <c r="N3" s="17" t="inlineStr">
         <is>
           <t>带锥度装置，适合斜度零件</t>
         </is>
       </c>
-      <c r="O3" s="10" t="inlineStr">
+      <c r="O3" s="16" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="4" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>SB-003</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>手摇平面磨床</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>TONVE-618</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>TONVE通伟</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>磨削设备</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="15" t="inlineStr">
         <is>
           <t>工作台150×450mm；砂轮直径180mm；手动进给</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="15" t="inlineStr">
         <is>
           <t>模具车间-磨削区</t>
         </is>
       </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="H4" s="16" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="I4" s="15" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="J4" s="15" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K4" s="10" t="inlineStr">
+      <c r="K4" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L4" s="10" t="inlineStr">
+      <c r="L4" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M4" s="9" t="inlineStr">
+      <c r="M4" s="15" t="inlineStr">
         <is>
           <t>砂轮防护罩/吸尘已配</t>
         </is>
       </c>
-      <c r="N4" s="11" t="inlineStr">
+      <c r="N4" s="17" t="inlineStr">
         <is>
           <t>配数显尺，精密小件磨削</t>
         </is>
       </c>
-      <c r="O4" s="10" t="inlineStr">
+      <c r="O4" s="16" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="5" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>SB-004</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>台式钻床</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>WMM-西菱</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>西菱WMM</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>钻削设备</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>最大钻孔直径16mm；工作台圆形；最大行程待补</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>模具车间-钳工台</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="H5" s="16" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I5" s="9" t="inlineStr">
+      <c r="I5" s="15" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J5" s="9" t="inlineStr">
+      <c r="J5" s="15" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K5" s="10" t="inlineStr">
+      <c r="K5" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L5" s="10" t="inlineStr">
+      <c r="L5" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M5" s="10" t="inlineStr">
+      <c r="M5" s="15" t="inlineStr">
         <is>
           <t>钻夹头钥匙/急停待确认</t>
         </is>
       </c>
-      <c r="N5" s="11" t="inlineStr">
+      <c r="N5" s="17" t="inlineStr">
         <is>
           <t>绿色机身，常规孔加工</t>
         </is>
       </c>
-      <c r="O5" s="10" t="inlineStr">
+      <c r="O5" s="16" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="6" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>SB-005</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>立式砂轮机</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>双工位砂轮机</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>磨削辅助设备</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>砂轮直径200mm；双砂轮（白刚玉+绿碳化硅）</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G6" s="15" t="inlineStr">
         <is>
           <t>模具车间-钳工角</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="16" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I6" s="9" t="inlineStr">
+      <c r="I6" s="15" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J6" s="9" t="inlineStr">
+      <c r="J6" s="15" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K6" s="10" t="inlineStr">
+      <c r="K6" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L6" s="10" t="inlineStr">
+      <c r="L6" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M6" s="9" t="inlineStr">
+      <c r="M6" s="15" t="inlineStr">
         <is>
           <t>砂轮防护罩/托架已配</t>
         </is>
       </c>
-      <c r="N6" s="11" t="inlineStr">
+      <c r="N6" s="17" t="inlineStr">
         <is>
           <t>磨刀/去毛刺专用</t>
         </is>
       </c>
-      <c r="O6" s="10" t="inlineStr">
+      <c r="O6" s="16" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="7" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>SB-006</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>台式电动冲床</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>JB04-1T</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>冲压设备</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="15" t="inlineStr">
         <is>
           <t>公称压力1吨；台式；手动按钮操作</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>模具车间-试模区</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H7" s="16" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I7" s="9" t="inlineStr">
+      <c r="I7" s="15" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J7" s="9" t="inlineStr">
+      <c r="J7" s="15" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K7" s="10" t="inlineStr">
+      <c r="K7" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L7" s="10" t="inlineStr">
+      <c r="L7" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M7" s="10" t="inlineStr">
+      <c r="M7" s="15" t="inlineStr">
         <is>
           <t>安全光幕/双手按钮待确认</t>
         </is>
       </c>
-      <c r="N7" s="11" t="inlineStr">
+      <c r="N7" s="17" t="inlineStr">
         <is>
           <t>小件试模、冲孔验证</t>
         </is>
       </c>
-      <c r="O7" s="10" t="inlineStr">
+      <c r="O7" s="16" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="8" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>SB-007</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>手摇平面磨床</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>SGM-450</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>曙光SHUGUANG</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
         <is>
           <t>磨削设备</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F8" s="15" t="inlineStr">
         <is>
           <t>工作台150×450mm；砂轮直径200mm；数显尺寸</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="G8" s="15" t="inlineStr">
         <is>
           <t>模具车间-磨削区</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="H8" s="16" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I8" s="9" t="inlineStr">
+      <c r="I8" s="15" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J8" s="9" t="inlineStr">
+      <c r="J8" s="15" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K8" s="10" t="inlineStr">
+      <c r="K8" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L8" s="10" t="inlineStr">
+      <c r="L8" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M8" s="9" t="inlineStr">
+      <c r="M8" s="15" t="inlineStr">
         <is>
           <t>砂轮防护罩/吸尘已配</t>
         </is>
       </c>
-      <c r="N8" s="11" t="inlineStr">
+      <c r="N8" s="17" t="inlineStr">
         <is>
           <t>与TONVE并排，配数显</t>
         </is>
       </c>
-      <c r="O8" s="10" t="inlineStr">
+      <c r="O8" s="16" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="9" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>SB-008</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>台式仪表车床</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>CJ0625B</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>恒生机床</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>车削设备</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t>最大回转直径250mm；最大加工长度300mm；手动进给</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>模具车间-钳工台旁</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I9" s="9" t="inlineStr">
+      <c r="I9" s="15" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J9" s="9" t="inlineStr">
+      <c r="J9" s="15" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K9" s="10" t="inlineStr">
+      <c r="K9" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L9" s="10" t="inlineStr">
+      <c r="L9" s="16" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M9" s="10" t="inlineStr">
+      <c r="M9" s="15" t="inlineStr">
         <is>
           <t>卡盘扳手/防护待确认</t>
         </is>
       </c>
-      <c r="N9" s="11" t="inlineStr">
+      <c r="N9" s="17" t="inlineStr">
         <is>
           <t>小件车削、螺纹加工</t>
         </is>
       </c>
-      <c r="O9" s="10" t="inlineStr">
+      <c r="O9" s="16" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
@@ -1412,10 +1399,9 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1426,115 +1412,126 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.466666666666667" defaultRowHeight="18.66666666666666"/>
   <cols>
-    <col width="23.66666666666667" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="23.66666666666667" customWidth="1" style="6" min="1" max="1"/>
+    <col width="110" customWidth="1" style="6" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>设备台账使用说明</t>
         </is>
       </c>
-      <c r="B1" s="12" t="n"/>
+      <c r="B1" s="18" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="n"/>
-      <c r="B2" s="13" t="n"/>
+      <c r="A2" s="15" t="n"/>
+      <c r="B2" s="15" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>1. 设备编号规则</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>SB-序号，按车间统一编号，一台一码，终身不变</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>2. 责任人</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>由生产主管指定，每台设备定岗到人</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>3. 当前状态</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>在用 / 待修 / 封存 / 报废</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>4. 保养等级</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>日点检（操作工）/ 周保养（班组长）/ 月保养（设备管理员）/ 年保养（外部）</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>5. 安全防护</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>开机前必须确认防护装置齐全有效</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>6. 备注</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>记录设备特殊用途、夹具、常用加工零件型号等</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="n"/>
-      <c r="B9" s="13" t="n"/>
+      <c r="A9" s="15" t="n"/>
+      <c r="B9" s="15" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>更新说明</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>本次为知识库设备台账更新优化：保留原有8条设备记录，增加筛选、表格化、下拉选项和核对状态；不将照片或现有文字当作最终铭牌/安全验收结论。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>配色说明</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>中国色取向：黛蓝用于表头和结构层级，朱砂用于待确认/待补，青黛用于来源/整理说明；所有浅色底均与文字颜色区分，确保可读性和黑白打印。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-10-29 12:29:56
</commit_message>
<xml_diff>
--- a/02_Areas/工作经历/鑫犇电子有限公司/01_生产部/工程技术组/设备台账.xlsx
+++ b/02_Areas/工作经历/鑫犇电子有限公司/01_生产部/工程技术组/设备台账.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -103,8 +103,25 @@
       <color rgb="00425066"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="00243B53"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <i val="1"/>
+      <color rgb="00007C91"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00102A43"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -136,8 +153,38 @@
         <fgColor rgb="00FCEDEA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00102A43"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B23A48"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F4F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B7791F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6F4F1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -155,11 +202,21 @@
         <color rgb="00425066"/>
       </bottom>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9E2EC"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00102A43"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -219,6 +276,39 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -693,693 +783,693 @@
   </cols>
   <sheetData>
     <row r="1" ht="37.33333333333333" customHeight="1" s="6">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>设备编号</t>
         </is>
       </c>
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="21" t="inlineStr">
         <is>
           <t>设备名称</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="21" t="inlineStr">
         <is>
           <t>型号规格</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="D1" s="21" t="inlineStr">
         <is>
           <t>品牌/产地</t>
         </is>
       </c>
-      <c r="E1" s="14" t="inlineStr">
+      <c r="E1" s="21" t="inlineStr">
         <is>
           <t>类别</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
+      <c r="F1" s="21" t="inlineStr">
         <is>
           <t>主要技术参数</t>
         </is>
       </c>
-      <c r="G1" s="14" t="inlineStr">
+      <c r="G1" s="21" t="inlineStr">
         <is>
           <t>工位位置</t>
         </is>
       </c>
-      <c r="H1" s="14" t="inlineStr">
+      <c r="H1" s="21" t="inlineStr">
         <is>
           <t>责任人</t>
         </is>
       </c>
-      <c r="I1" s="14" t="inlineStr">
+      <c r="I1" s="21" t="inlineStr">
         <is>
           <t>当前状态</t>
         </is>
       </c>
-      <c r="J1" s="14" t="inlineStr">
+      <c r="J1" s="21" t="inlineStr">
         <is>
           <t>保养等级</t>
         </is>
       </c>
-      <c r="K1" s="14" t="inlineStr">
+      <c r="K1" s="21" t="inlineStr">
         <is>
           <t>上次保养</t>
         </is>
       </c>
-      <c r="L1" s="14" t="inlineStr">
+      <c r="L1" s="21" t="inlineStr">
         <is>
           <t>下次保养</t>
         </is>
       </c>
-      <c r="M1" s="14" t="inlineStr">
+      <c r="M1" s="21" t="inlineStr">
         <is>
           <t>安全防护</t>
         </is>
       </c>
-      <c r="N1" s="14" t="inlineStr">
+      <c r="N1" s="21" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="O1" s="14" t="inlineStr">
+      <c r="O1" s="21" t="inlineStr">
         <is>
           <t>核对状态</t>
         </is>
       </c>
     </row>
     <row r="2" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>SB-001</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="B2" s="22" t="inlineStr">
         <is>
           <t>快走丝线切割</t>
         </is>
       </c>
-      <c r="C2" s="15" t="inlineStr">
+      <c r="C2" s="22" t="inlineStr">
         <is>
           <t>DK7732</t>
         </is>
       </c>
-      <c r="D2" s="15" t="inlineStr">
+      <c r="D2" s="22" t="inlineStr">
         <is>
           <t>泰州四海数控</t>
         </is>
       </c>
-      <c r="E2" s="15" t="inlineStr">
+      <c r="E2" s="22" t="inlineStr">
         <is>
           <t>电加工设备</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
+      <c r="F2" s="22" t="inlineStr">
         <is>
           <t>最大加工厚度300mm；锥度±3°；工作台行程320×400mm</t>
         </is>
       </c>
-      <c r="G2" s="15" t="inlineStr">
+      <c r="G2" s="22" t="inlineStr">
         <is>
           <t>模具车间-线切割区</t>
         </is>
       </c>
-      <c r="H2" s="16" t="inlineStr">
+      <c r="H2" s="23" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I2" s="15" t="inlineStr">
+      <c r="I2" s="22" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J2" s="15" t="inlineStr">
+      <c r="J2" s="22" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K2" s="16" t="inlineStr">
+      <c r="K2" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L2" s="16" t="inlineStr">
+      <c r="L2" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M2" s="15" t="inlineStr">
+      <c r="M2" s="22" t="inlineStr">
         <is>
           <t>防护门/急停已配</t>
         </is>
       </c>
-      <c r="N2" s="17" t="inlineStr">
+      <c r="N2" s="24" t="inlineStr">
         <is>
           <t>双机位油槽，带数控系统</t>
         </is>
       </c>
-      <c r="O2" s="16" t="inlineStr">
+      <c r="O2" s="23" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="3" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>SB-002</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
+      <c r="B3" s="25" t="inlineStr">
         <is>
           <t>锥度线切割</t>
         </is>
       </c>
-      <c r="C3" s="15" t="inlineStr">
+      <c r="C3" s="25" t="inlineStr">
         <is>
           <t>DK7735</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
+      <c r="D3" s="25" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E3" s="15" t="inlineStr">
+      <c r="E3" s="25" t="inlineStr">
         <is>
           <t>电加工设备</t>
         </is>
       </c>
-      <c r="F3" s="15" t="inlineStr">
+      <c r="F3" s="25" t="inlineStr">
         <is>
           <t>最大加工厚度350mm；大锥度切割；工作台行程350×500mm</t>
         </is>
       </c>
-      <c r="G3" s="15" t="inlineStr">
+      <c r="G3" s="25" t="inlineStr">
         <is>
           <t>模具车间-线切割区</t>
         </is>
       </c>
-      <c r="H3" s="16" t="inlineStr">
+      <c r="H3" s="23" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I3" s="15" t="inlineStr">
+      <c r="I3" s="25" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J3" s="15" t="inlineStr">
+      <c r="J3" s="25" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K3" s="16" t="inlineStr">
+      <c r="K3" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L3" s="16" t="inlineStr">
+      <c r="L3" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M3" s="15" t="inlineStr">
+      <c r="M3" s="25" t="inlineStr">
         <is>
           <t>防护门/急停已配</t>
         </is>
       </c>
-      <c r="N3" s="17" t="inlineStr">
+      <c r="N3" s="26" t="inlineStr">
         <is>
           <t>带锥度装置，适合斜度零件</t>
         </is>
       </c>
-      <c r="O3" s="16" t="inlineStr">
+      <c r="O3" s="23" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="4" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>SB-003</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>手摇平面磨床</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>TONVE-618</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="22" t="inlineStr">
         <is>
           <t>TONVE通伟</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="22" t="inlineStr">
         <is>
           <t>磨削设备</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr">
+      <c r="F4" s="22" t="inlineStr">
         <is>
           <t>工作台150×450mm；砂轮直径180mm；手动进给</t>
         </is>
       </c>
-      <c r="G4" s="15" t="inlineStr">
+      <c r="G4" s="22" t="inlineStr">
         <is>
           <t>模具车间-磨削区</t>
         </is>
       </c>
-      <c r="H4" s="16" t="inlineStr">
+      <c r="H4" s="23" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I4" s="15" t="inlineStr">
+      <c r="I4" s="22" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J4" s="15" t="inlineStr">
+      <c r="J4" s="22" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K4" s="16" t="inlineStr">
+      <c r="K4" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L4" s="16" t="inlineStr">
+      <c r="L4" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M4" s="15" t="inlineStr">
+      <c r="M4" s="22" t="inlineStr">
         <is>
           <t>砂轮防护罩/吸尘已配</t>
         </is>
       </c>
-      <c r="N4" s="17" t="inlineStr">
+      <c r="N4" s="24" t="inlineStr">
         <is>
           <t>配数显尺，精密小件磨削</t>
         </is>
       </c>
-      <c r="O4" s="16" t="inlineStr">
+      <c r="O4" s="23" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="5" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>SB-004</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>台式钻床</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>WMM-西菱</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>西菱WMM</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>钻削设备</t>
         </is>
       </c>
-      <c r="F5" s="15" t="inlineStr">
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>最大钻孔直径16mm；工作台圆形；最大行程待补</t>
         </is>
       </c>
-      <c r="G5" s="15" t="inlineStr">
+      <c r="G5" s="25" t="inlineStr">
         <is>
           <t>模具车间-钳工台</t>
         </is>
       </c>
-      <c r="H5" s="16" t="inlineStr">
+      <c r="H5" s="23" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I5" s="15" t="inlineStr">
+      <c r="I5" s="25" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J5" s="15" t="inlineStr">
+      <c r="J5" s="25" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K5" s="16" t="inlineStr">
+      <c r="K5" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L5" s="16" t="inlineStr">
+      <c r="L5" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M5" s="15" t="inlineStr">
+      <c r="M5" s="27" t="inlineStr">
         <is>
           <t>钻夹头钥匙/急停待确认</t>
         </is>
       </c>
-      <c r="N5" s="17" t="inlineStr">
+      <c r="N5" s="26" t="inlineStr">
         <is>
           <t>绿色机身，常规孔加工</t>
         </is>
       </c>
-      <c r="O5" s="16" t="inlineStr">
+      <c r="O5" s="23" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="6" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>SB-005</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>立式砂轮机</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>双工位砂轮机</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>磨削辅助设备</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="22" t="inlineStr">
         <is>
           <t>砂轮直径200mm；双砂轮（白刚玉+绿碳化硅）</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="22" t="inlineStr">
         <is>
           <t>模具车间-钳工角</t>
         </is>
       </c>
-      <c r="H6" s="16" t="inlineStr">
+      <c r="H6" s="23" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I6" s="15" t="inlineStr">
+      <c r="I6" s="22" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J6" s="15" t="inlineStr">
+      <c r="J6" s="22" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K6" s="16" t="inlineStr">
+      <c r="K6" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L6" s="16" t="inlineStr">
+      <c r="L6" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M6" s="15" t="inlineStr">
+      <c r="M6" s="22" t="inlineStr">
         <is>
           <t>砂轮防护罩/托架已配</t>
         </is>
       </c>
-      <c r="N6" s="17" t="inlineStr">
+      <c r="N6" s="24" t="inlineStr">
         <is>
           <t>磨刀/去毛刺专用</t>
         </is>
       </c>
-      <c r="O6" s="16" t="inlineStr">
+      <c r="O6" s="23" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="7" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>SB-006</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="25" t="inlineStr">
         <is>
           <t>台式电动冲床</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>JB04-1T</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="D7" s="25" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E7" s="15" t="inlineStr">
+      <c r="E7" s="25" t="inlineStr">
         <is>
           <t>冲压设备</t>
         </is>
       </c>
-      <c r="F7" s="15" t="inlineStr">
+      <c r="F7" s="25" t="inlineStr">
         <is>
           <t>公称压力1吨；台式；手动按钮操作</t>
         </is>
       </c>
-      <c r="G7" s="15" t="inlineStr">
+      <c r="G7" s="25" t="inlineStr">
         <is>
           <t>模具车间-试模区</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="23" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I7" s="15" t="inlineStr">
+      <c r="I7" s="25" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J7" s="15" t="inlineStr">
+      <c r="J7" s="25" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K7" s="16" t="inlineStr">
+      <c r="K7" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L7" s="16" t="inlineStr">
+      <c r="L7" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M7" s="15" t="inlineStr">
+      <c r="M7" s="27" t="inlineStr">
         <is>
           <t>安全光幕/双手按钮待确认</t>
         </is>
       </c>
-      <c r="N7" s="17" t="inlineStr">
+      <c r="N7" s="26" t="inlineStr">
         <is>
           <t>小件试模、冲孔验证</t>
         </is>
       </c>
-      <c r="O7" s="16" t="inlineStr">
+      <c r="O7" s="23" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="8" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>SB-007</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>手摇平面磨床</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>SGM-450</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>曙光SHUGUANG</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>磨削设备</t>
         </is>
       </c>
-      <c r="F8" s="15" t="inlineStr">
+      <c r="F8" s="22" t="inlineStr">
         <is>
           <t>工作台150×450mm；砂轮直径200mm；数显尺寸</t>
         </is>
       </c>
-      <c r="G8" s="15" t="inlineStr">
+      <c r="G8" s="22" t="inlineStr">
         <is>
           <t>模具车间-磨削区</t>
         </is>
       </c>
-      <c r="H8" s="16" t="inlineStr">
+      <c r="H8" s="23" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I8" s="15" t="inlineStr">
+      <c r="I8" s="22" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J8" s="15" t="inlineStr">
+      <c r="J8" s="22" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K8" s="16" t="inlineStr">
+      <c r="K8" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L8" s="16" t="inlineStr">
+      <c r="L8" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M8" s="15" t="inlineStr">
+      <c r="M8" s="22" t="inlineStr">
         <is>
           <t>砂轮防护罩/吸尘已配</t>
         </is>
       </c>
-      <c r="N8" s="17" t="inlineStr">
+      <c r="N8" s="24" t="inlineStr">
         <is>
           <t>与TONVE并排，配数显</t>
         </is>
       </c>
-      <c r="O8" s="16" t="inlineStr">
+      <c r="O8" s="23" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="9" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>SB-008</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="25" t="inlineStr">
         <is>
           <t>台式仪表车床</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
         <is>
           <t>CJ0625B</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="25" t="inlineStr">
         <is>
           <t>恒生机床</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="25" t="inlineStr">
         <is>
           <t>车削设备</t>
         </is>
       </c>
-      <c r="F9" s="15" t="inlineStr">
+      <c r="F9" s="25" t="inlineStr">
         <is>
           <t>最大回转直径250mm；最大加工长度300mm；手动进给</t>
         </is>
       </c>
-      <c r="G9" s="15" t="inlineStr">
+      <c r="G9" s="25" t="inlineStr">
         <is>
           <t>模具车间-钳工台旁</t>
         </is>
       </c>
-      <c r="H9" s="16" t="inlineStr">
+      <c r="H9" s="23" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I9" s="15" t="inlineStr">
+      <c r="I9" s="25" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J9" s="15" t="inlineStr">
+      <c r="J9" s="25" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K9" s="16" t="inlineStr">
+      <c r="K9" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L9" s="16" t="inlineStr">
+      <c r="L9" s="23" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M9" s="15" t="inlineStr">
+      <c r="M9" s="27" t="inlineStr">
         <is>
           <t>卡盘扳手/防护待确认</t>
         </is>
       </c>
-      <c r="N9" s="17" t="inlineStr">
+      <c r="N9" s="26" t="inlineStr">
         <is>
           <t>小件车削、螺纹加工</t>
         </is>
       </c>
-      <c r="O9" s="16" t="inlineStr">
+      <c r="O9" s="23" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
@@ -1420,114 +1510,114 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>设备台账使用说明</t>
         </is>
       </c>
-      <c r="B1" s="18" t="n"/>
+      <c r="B1" s="28" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="n"/>
-      <c r="B2" s="15" t="n"/>
+      <c r="A2" s="29" t="n"/>
+      <c r="B2" s="29" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="29" t="inlineStr">
         <is>
           <t>1. 设备编号规则</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
+      <c r="B3" s="29" t="inlineStr">
         <is>
           <t>SB-序号，按车间统一编号，一台一码，终身不变</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>2. 责任人</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>由生产主管指定，每台设备定岗到人</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>3. 当前状态</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>在用 / 待修 / 封存 / 报废</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>4. 保养等级</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>日点检（操作工）/ 周保养（班组长）/ 月保养（设备管理员）/ 年保养（外部）</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>5. 安全防护</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>开机前必须确认防护装置齐全有效</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>6. 备注</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>记录设备特殊用途、夹具、常用加工零件型号等</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="n"/>
-      <c r="B9" s="15" t="n"/>
+      <c r="A9" s="29" t="n"/>
+      <c r="B9" s="29" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>更新说明</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="29" t="inlineStr">
         <is>
           <t>本次为知识库设备台账更新优化：保留原有8条设备记录，增加筛选、表格化、下拉选项和核对状态；不将照片或现有文字当作最终铭牌/安全验收结论。</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>配色说明</t>
-        </is>
-      </c>
-      <c r="B11" s="20" t="inlineStr">
-        <is>
-          <t>中国色取向：黛蓝用于表头和结构层级，朱砂用于待确认/待补，青黛用于来源/整理说明；所有浅色底均与文字颜色区分，确保可读性和黑白打印。</t>
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>配色规范</t>
+        </is>
+      </c>
+      <c r="B11" s="31" t="inlineStr">
+        <is>
+          <t>国际企业管理系统风格：深海军蓝（结构/表头）+ 青绿色（来源/说明）+ 琥珀金（安全关注）+ 朱红（待确认/待补/异常）。���色底统一使用白字，正文使用墨色；不使用同色底与同色字。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-10-29 12:40:34
</commit_message>
<xml_diff>
--- a/02_Areas/工作经历/鑫犇电子有限公司/01_生产部/工程技术组/设备台账.xlsx
+++ b/02_Areas/工作经历/鑫犇电子有限公司/01_生产部/工程技术组/设备台账.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -120,8 +120,37 @@
       <color rgb="00102A43"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="001D1D1F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="001D1D1F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <i val="1"/>
+      <color rgb="000071E3"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00FF3B30"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00FF9F0A"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -183,8 +212,23 @@
         <fgColor rgb="00E6F4F1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F9FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAFAFC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -212,11 +256,21 @@
         <color rgb="00102A43"/>
       </bottom>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D2D2D7"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="000071E3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -309,6 +363,36 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -782,694 +866,694 @@
     <col width="16" customWidth="1" style="6" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="37.33333333333333" customHeight="1" s="6">
-      <c r="A1" s="21" t="inlineStr">
+    <row r="1" ht="28" customHeight="1" s="6">
+      <c r="A1" s="32" t="inlineStr">
         <is>
           <t>设备编号</t>
         </is>
       </c>
-      <c r="B1" s="21" t="inlineStr">
+      <c r="B1" s="32" t="inlineStr">
         <is>
           <t>设备名称</t>
         </is>
       </c>
-      <c r="C1" s="21" t="inlineStr">
+      <c r="C1" s="32" t="inlineStr">
         <is>
           <t>型号规格</t>
         </is>
       </c>
-      <c r="D1" s="21" t="inlineStr">
+      <c r="D1" s="32" t="inlineStr">
         <is>
           <t>品牌/产地</t>
         </is>
       </c>
-      <c r="E1" s="21" t="inlineStr">
+      <c r="E1" s="32" t="inlineStr">
         <is>
           <t>类别</t>
         </is>
       </c>
-      <c r="F1" s="21" t="inlineStr">
+      <c r="F1" s="32" t="inlineStr">
         <is>
           <t>主要技术参数</t>
         </is>
       </c>
-      <c r="G1" s="21" t="inlineStr">
+      <c r="G1" s="32" t="inlineStr">
         <is>
           <t>工位位置</t>
         </is>
       </c>
-      <c r="H1" s="21" t="inlineStr">
+      <c r="H1" s="32" t="inlineStr">
         <is>
           <t>责任人</t>
         </is>
       </c>
-      <c r="I1" s="21" t="inlineStr">
+      <c r="I1" s="32" t="inlineStr">
         <is>
           <t>当前状态</t>
         </is>
       </c>
-      <c r="J1" s="21" t="inlineStr">
+      <c r="J1" s="32" t="inlineStr">
         <is>
           <t>保养等级</t>
         </is>
       </c>
-      <c r="K1" s="21" t="inlineStr">
+      <c r="K1" s="32" t="inlineStr">
         <is>
           <t>上次保养</t>
         </is>
       </c>
-      <c r="L1" s="21" t="inlineStr">
+      <c r="L1" s="32" t="inlineStr">
         <is>
           <t>下次保养</t>
         </is>
       </c>
-      <c r="M1" s="21" t="inlineStr">
+      <c r="M1" s="32" t="inlineStr">
         <is>
           <t>安全防护</t>
         </is>
       </c>
-      <c r="N1" s="21" t="inlineStr">
+      <c r="N1" s="32" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="O1" s="21" t="inlineStr">
+      <c r="O1" s="32" t="inlineStr">
         <is>
           <t>核对状态</t>
         </is>
       </c>
     </row>
     <row r="2" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="33" t="inlineStr">
         <is>
           <t>SB-001</t>
         </is>
       </c>
-      <c r="B2" s="22" t="inlineStr">
+      <c r="B2" s="33" t="inlineStr">
         <is>
           <t>快走丝线切割</t>
         </is>
       </c>
-      <c r="C2" s="22" t="inlineStr">
+      <c r="C2" s="33" t="inlineStr">
         <is>
           <t>DK7732</t>
         </is>
       </c>
-      <c r="D2" s="22" t="inlineStr">
+      <c r="D2" s="33" t="inlineStr">
         <is>
           <t>泰州四海数控</t>
         </is>
       </c>
-      <c r="E2" s="22" t="inlineStr">
+      <c r="E2" s="33" t="inlineStr">
         <is>
           <t>电加工设备</t>
         </is>
       </c>
-      <c r="F2" s="22" t="inlineStr">
+      <c r="F2" s="33" t="inlineStr">
         <is>
           <t>最大加工厚度300mm；锥度±3°；工作台行程320×400mm</t>
         </is>
       </c>
-      <c r="G2" s="22" t="inlineStr">
+      <c r="G2" s="33" t="inlineStr">
         <is>
           <t>模具车间-线切割区</t>
         </is>
       </c>
-      <c r="H2" s="23" t="inlineStr">
+      <c r="H2" s="34" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I2" s="22" t="inlineStr">
+      <c r="I2" s="33" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J2" s="22" t="inlineStr">
+      <c r="J2" s="33" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K2" s="23" t="inlineStr">
+      <c r="K2" s="34" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L2" s="23" t="inlineStr">
+      <c r="L2" s="34" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M2" s="22" t="inlineStr">
+      <c r="M2" s="33" t="inlineStr">
         <is>
           <t>防护门/急停已配</t>
         </is>
       </c>
-      <c r="N2" s="24" t="inlineStr">
+      <c r="N2" s="35" t="inlineStr">
         <is>
           <t>双机位油槽，带数控系统</t>
         </is>
       </c>
-      <c r="O2" s="23" t="inlineStr">
+      <c r="O2" s="34" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="3" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A3" s="25" t="inlineStr">
+      <c r="A3" s="36" t="inlineStr">
         <is>
           <t>SB-002</t>
         </is>
       </c>
-      <c r="B3" s="25" t="inlineStr">
+      <c r="B3" s="36" t="inlineStr">
         <is>
           <t>锥度线切割</t>
         </is>
       </c>
-      <c r="C3" s="25" t="inlineStr">
+      <c r="C3" s="36" t="inlineStr">
         <is>
           <t>DK7735</t>
         </is>
       </c>
-      <c r="D3" s="25" t="inlineStr">
+      <c r="D3" s="36" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E3" s="25" t="inlineStr">
+      <c r="E3" s="36" t="inlineStr">
         <is>
           <t>电加工设备</t>
         </is>
       </c>
-      <c r="F3" s="25" t="inlineStr">
+      <c r="F3" s="36" t="inlineStr">
         <is>
           <t>最大加工厚度350mm；大锥度切割；工作台行程350×500mm</t>
         </is>
       </c>
-      <c r="G3" s="25" t="inlineStr">
+      <c r="G3" s="36" t="inlineStr">
         <is>
           <t>模具车间-线切割区</t>
         </is>
       </c>
-      <c r="H3" s="23" t="inlineStr">
+      <c r="H3" s="37" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I3" s="25" t="inlineStr">
+      <c r="I3" s="36" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J3" s="25" t="inlineStr">
+      <c r="J3" s="36" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K3" s="23" t="inlineStr">
+      <c r="K3" s="37" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L3" s="23" t="inlineStr">
+      <c r="L3" s="37" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M3" s="25" t="inlineStr">
+      <c r="M3" s="36" t="inlineStr">
         <is>
           <t>防护门/急停已配</t>
         </is>
       </c>
-      <c r="N3" s="26" t="inlineStr">
+      <c r="N3" s="35" t="inlineStr">
         <is>
           <t>带锥度装置，适合斜度零件</t>
         </is>
       </c>
-      <c r="O3" s="23" t="inlineStr">
+      <c r="O3" s="37" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="4" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="33" t="inlineStr">
         <is>
           <t>SB-003</t>
         </is>
       </c>
-      <c r="B4" s="22" t="inlineStr">
+      <c r="B4" s="33" t="inlineStr">
         <is>
           <t>手摇平面磨床</t>
         </is>
       </c>
-      <c r="C4" s="22" t="inlineStr">
+      <c r="C4" s="33" t="inlineStr">
         <is>
           <t>TONVE-618</t>
         </is>
       </c>
-      <c r="D4" s="22" t="inlineStr">
+      <c r="D4" s="33" t="inlineStr">
         <is>
           <t>TONVE通伟</t>
         </is>
       </c>
-      <c r="E4" s="22" t="inlineStr">
+      <c r="E4" s="33" t="inlineStr">
         <is>
           <t>磨削设备</t>
         </is>
       </c>
-      <c r="F4" s="22" t="inlineStr">
+      <c r="F4" s="33" t="inlineStr">
         <is>
           <t>工作台150×450mm；砂轮直径180mm；手动进给</t>
         </is>
       </c>
-      <c r="G4" s="22" t="inlineStr">
+      <c r="G4" s="33" t="inlineStr">
         <is>
           <t>模具车间-磨削区</t>
         </is>
       </c>
-      <c r="H4" s="23" t="inlineStr">
+      <c r="H4" s="34" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I4" s="22" t="inlineStr">
+      <c r="I4" s="33" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J4" s="22" t="inlineStr">
+      <c r="J4" s="33" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K4" s="23" t="inlineStr">
+      <c r="K4" s="34" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L4" s="23" t="inlineStr">
+      <c r="L4" s="34" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M4" s="22" t="inlineStr">
+      <c r="M4" s="33" t="inlineStr">
         <is>
           <t>砂轮防护罩/吸尘已配</t>
         </is>
       </c>
-      <c r="N4" s="24" t="inlineStr">
+      <c r="N4" s="35" t="inlineStr">
         <is>
           <t>配数显尺，精密小件磨削</t>
         </is>
       </c>
-      <c r="O4" s="23" t="inlineStr">
+      <c r="O4" s="34" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="5" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="36" t="inlineStr">
         <is>
           <t>SB-004</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="36" t="inlineStr">
         <is>
           <t>台式钻床</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="36" t="inlineStr">
         <is>
           <t>WMM-西菱</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="36" t="inlineStr">
         <is>
           <t>西菱WMM</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="36" t="inlineStr">
         <is>
           <t>钻削设备</t>
         </is>
       </c>
-      <c r="F5" s="25" t="inlineStr">
+      <c r="F5" s="36" t="inlineStr">
         <is>
           <t>最大钻孔直径16mm；工作台圆形；最大行程待补</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="G5" s="36" t="inlineStr">
         <is>
           <t>模具车间-钳工台</t>
         </is>
       </c>
-      <c r="H5" s="23" t="inlineStr">
+      <c r="H5" s="37" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I5" s="25" t="inlineStr">
+      <c r="I5" s="36" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J5" s="25" t="inlineStr">
+      <c r="J5" s="36" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K5" s="23" t="inlineStr">
+      <c r="K5" s="37" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L5" s="23" t="inlineStr">
+      <c r="L5" s="37" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M5" s="27" t="inlineStr">
+      <c r="M5" s="38" t="inlineStr">
         <is>
           <t>钻夹头钥匙/急停待确认</t>
         </is>
       </c>
-      <c r="N5" s="26" t="inlineStr">
+      <c r="N5" s="35" t="inlineStr">
         <is>
           <t>绿色机身，常规孔加工</t>
         </is>
       </c>
-      <c r="O5" s="23" t="inlineStr">
+      <c r="O5" s="37" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="6" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="33" t="inlineStr">
         <is>
           <t>SB-005</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
+      <c r="B6" s="33" t="inlineStr">
         <is>
           <t>立式砂轮机</t>
         </is>
       </c>
-      <c r="C6" s="22" t="inlineStr">
+      <c r="C6" s="33" t="inlineStr">
         <is>
           <t>双工位砂轮机</t>
         </is>
       </c>
-      <c r="D6" s="22" t="inlineStr">
+      <c r="D6" s="33" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E6" s="22" t="inlineStr">
+      <c r="E6" s="33" t="inlineStr">
         <is>
           <t>磨削辅助设备</t>
         </is>
       </c>
-      <c r="F6" s="22" t="inlineStr">
+      <c r="F6" s="33" t="inlineStr">
         <is>
           <t>砂轮直径200mm；双砂轮（白刚玉+绿碳化硅）</t>
         </is>
       </c>
-      <c r="G6" s="22" t="inlineStr">
+      <c r="G6" s="33" t="inlineStr">
         <is>
           <t>模具车间-钳工角</t>
         </is>
       </c>
-      <c r="H6" s="23" t="inlineStr">
+      <c r="H6" s="34" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I6" s="22" t="inlineStr">
+      <c r="I6" s="33" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J6" s="22" t="inlineStr">
+      <c r="J6" s="33" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K6" s="23" t="inlineStr">
+      <c r="K6" s="34" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L6" s="23" t="inlineStr">
+      <c r="L6" s="34" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M6" s="22" t="inlineStr">
+      <c r="M6" s="33" t="inlineStr">
         <is>
           <t>砂轮防护罩/托架已配</t>
         </is>
       </c>
-      <c r="N6" s="24" t="inlineStr">
+      <c r="N6" s="35" t="inlineStr">
         <is>
           <t>磨刀/去毛刺专用</t>
         </is>
       </c>
-      <c r="O6" s="23" t="inlineStr">
+      <c r="O6" s="34" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="7" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="36" t="inlineStr">
         <is>
           <t>SB-006</t>
         </is>
       </c>
-      <c r="B7" s="25" t="inlineStr">
+      <c r="B7" s="36" t="inlineStr">
         <is>
           <t>台式电动冲床</t>
         </is>
       </c>
-      <c r="C7" s="25" t="inlineStr">
+      <c r="C7" s="36" t="inlineStr">
         <is>
           <t>JB04-1T</t>
         </is>
       </c>
-      <c r="D7" s="25" t="inlineStr">
+      <c r="D7" s="36" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E7" s="25" t="inlineStr">
+      <c r="E7" s="36" t="inlineStr">
         <is>
           <t>冲压设备</t>
         </is>
       </c>
-      <c r="F7" s="25" t="inlineStr">
+      <c r="F7" s="36" t="inlineStr">
         <is>
           <t>公称压力1吨；台式；手动按钮操作</t>
         </is>
       </c>
-      <c r="G7" s="25" t="inlineStr">
+      <c r="G7" s="36" t="inlineStr">
         <is>
           <t>模具车间-试模区</t>
         </is>
       </c>
-      <c r="H7" s="23" t="inlineStr">
+      <c r="H7" s="37" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I7" s="25" t="inlineStr">
+      <c r="I7" s="36" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J7" s="25" t="inlineStr">
+      <c r="J7" s="36" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K7" s="23" t="inlineStr">
+      <c r="K7" s="37" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L7" s="23" t="inlineStr">
+      <c r="L7" s="37" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M7" s="27" t="inlineStr">
+      <c r="M7" s="38" t="inlineStr">
         <is>
           <t>安全光幕/双手按钮待确认</t>
         </is>
       </c>
-      <c r="N7" s="26" t="inlineStr">
+      <c r="N7" s="35" t="inlineStr">
         <is>
           <t>小件试模、冲孔验证</t>
         </is>
       </c>
-      <c r="O7" s="23" t="inlineStr">
+      <c r="O7" s="37" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="8" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="33" t="inlineStr">
         <is>
           <t>SB-007</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="33" t="inlineStr">
         <is>
           <t>手摇平面磨床</t>
         </is>
       </c>
-      <c r="C8" s="22" t="inlineStr">
+      <c r="C8" s="33" t="inlineStr">
         <is>
           <t>SGM-450</t>
         </is>
       </c>
-      <c r="D8" s="22" t="inlineStr">
+      <c r="D8" s="33" t="inlineStr">
         <is>
           <t>曙光SHUGUANG</t>
         </is>
       </c>
-      <c r="E8" s="22" t="inlineStr">
+      <c r="E8" s="33" t="inlineStr">
         <is>
           <t>磨削设备</t>
         </is>
       </c>
-      <c r="F8" s="22" t="inlineStr">
+      <c r="F8" s="33" t="inlineStr">
         <is>
           <t>工作台150×450mm；砂轮直径200mm；数显尺寸</t>
         </is>
       </c>
-      <c r="G8" s="22" t="inlineStr">
+      <c r="G8" s="33" t="inlineStr">
         <is>
           <t>模具车间-磨削区</t>
         </is>
       </c>
-      <c r="H8" s="23" t="inlineStr">
+      <c r="H8" s="34" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I8" s="22" t="inlineStr">
+      <c r="I8" s="33" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J8" s="22" t="inlineStr">
+      <c r="J8" s="33" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K8" s="23" t="inlineStr">
+      <c r="K8" s="34" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L8" s="23" t="inlineStr">
+      <c r="L8" s="34" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M8" s="22" t="inlineStr">
+      <c r="M8" s="33" t="inlineStr">
         <is>
           <t>砂轮防护罩/吸尘已配</t>
         </is>
       </c>
-      <c r="N8" s="24" t="inlineStr">
+      <c r="N8" s="35" t="inlineStr">
         <is>
           <t>与TONVE并排，配数显</t>
         </is>
       </c>
-      <c r="O8" s="23" t="inlineStr">
+      <c r="O8" s="34" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="9" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A9" s="25" t="inlineStr">
+      <c r="A9" s="36" t="inlineStr">
         <is>
           <t>SB-008</t>
         </is>
       </c>
-      <c r="B9" s="25" t="inlineStr">
+      <c r="B9" s="36" t="inlineStr">
         <is>
           <t>台式仪表车床</t>
         </is>
       </c>
-      <c r="C9" s="25" t="inlineStr">
+      <c r="C9" s="36" t="inlineStr">
         <is>
           <t>CJ0625B</t>
         </is>
       </c>
-      <c r="D9" s="25" t="inlineStr">
+      <c r="D9" s="36" t="inlineStr">
         <is>
           <t>恒生机床</t>
         </is>
       </c>
-      <c r="E9" s="25" t="inlineStr">
+      <c r="E9" s="36" t="inlineStr">
         <is>
           <t>车削设备</t>
         </is>
       </c>
-      <c r="F9" s="25" t="inlineStr">
+      <c r="F9" s="36" t="inlineStr">
         <is>
           <t>最大回转直径250mm；最大加工长度300mm；手动进给</t>
         </is>
       </c>
-      <c r="G9" s="25" t="inlineStr">
+      <c r="G9" s="36" t="inlineStr">
         <is>
           <t>模具车间-钳工台旁</t>
         </is>
       </c>
-      <c r="H9" s="23" t="inlineStr">
+      <c r="H9" s="37" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I9" s="25" t="inlineStr">
+      <c r="I9" s="36" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J9" s="25" t="inlineStr">
+      <c r="J9" s="36" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K9" s="23" t="inlineStr">
+      <c r="K9" s="37" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L9" s="23" t="inlineStr">
+      <c r="L9" s="37" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M9" s="27" t="inlineStr">
+      <c r="M9" s="38" t="inlineStr">
         <is>
           <t>卡盘扳手/防护待确认</t>
         </is>
       </c>
-      <c r="N9" s="26" t="inlineStr">
+      <c r="N9" s="35" t="inlineStr">
         <is>
           <t>小件车削、螺纹加工</t>
         </is>
       </c>
-      <c r="O9" s="23" t="inlineStr">
+      <c r="O9" s="37" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
@@ -1510,114 +1594,114 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="39" t="inlineStr">
         <is>
           <t>设备台账使用说明</t>
         </is>
       </c>
-      <c r="B1" s="28" t="n"/>
+      <c r="B1" s="39" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="29" t="n"/>
-      <c r="B2" s="29" t="n"/>
+      <c r="A2" s="40" t="n"/>
+      <c r="B2" s="40" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="29" t="inlineStr">
+      <c r="A3" s="40" t="inlineStr">
         <is>
           <t>1. 设备编号规则</t>
         </is>
       </c>
-      <c r="B3" s="29" t="inlineStr">
+      <c r="B3" s="40" t="inlineStr">
         <is>
           <t>SB-序号，按车间统一编号，一台一码，终身不变</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="40" t="inlineStr">
         <is>
           <t>2. 责任人</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="B4" s="40" t="inlineStr">
         <is>
           <t>由生产主管指定，每台设备定岗到人</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="inlineStr">
+      <c r="A5" s="40" t="inlineStr">
         <is>
           <t>3. 当前状态</t>
         </is>
       </c>
-      <c r="B5" s="29" t="inlineStr">
+      <c r="B5" s="40" t="inlineStr">
         <is>
           <t>在用 / 待修 / 封存 / 报废</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="40" t="inlineStr">
         <is>
           <t>4. 保养等级</t>
         </is>
       </c>
-      <c r="B6" s="29" t="inlineStr">
+      <c r="B6" s="40" t="inlineStr">
         <is>
           <t>日点检（操作工）/ 周保养（班组长）/ 月保养（设备管理员）/ 年保养（外部）</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="29" t="inlineStr">
+      <c r="A7" s="40" t="inlineStr">
         <is>
           <t>5. 安全防护</t>
         </is>
       </c>
-      <c r="B7" s="29" t="inlineStr">
+      <c r="B7" s="40" t="inlineStr">
         <is>
           <t>开机前必须确认防护装置齐全有效</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="40" t="inlineStr">
         <is>
           <t>6. 备注</t>
         </is>
       </c>
-      <c r="B8" s="29" t="inlineStr">
+      <c r="B8" s="40" t="inlineStr">
         <is>
           <t>记录设备特殊用途、夹具、常用加工零件型号等</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="n"/>
-      <c r="B9" s="29" t="n"/>
+      <c r="A9" s="40" t="n"/>
+      <c r="B9" s="40" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="40" t="inlineStr">
         <is>
           <t>更新说明</t>
         </is>
       </c>
-      <c r="B10" s="29" t="inlineStr">
+      <c r="B10" s="40" t="inlineStr">
         <is>
           <t>本次为知识库设备台账更新优化：保留原有8条设备记录，增加筛选、表格化、下拉选项和核对状态；不将照片或现有文字当作最终铭牌/安全验收结论。</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="41" t="inlineStr">
         <is>
           <t>配色规范</t>
         </is>
       </c>
-      <c r="B11" s="31" t="inlineStr">
-        <is>
-          <t>国际企业管理系统风格：深海军蓝（结构/表头）+ 青绿色（来源/说明）+ 琥珀金（安全关注）+ 朱红（待确认/待补/异常）。���色底统一使用白字，正文使用墨色；不使用同色底与同色字。</t>
+      <c r="B11" s="35" t="inlineStr">
+        <is>
+          <t>苹果式浅色界面取向：白色/极浅灰为主，深灰为正文，系统蓝仅作结构强调，红色仅表示待确认/待补，橙色仅表示安全关注；不使用大面积深色底、不使用同色底字。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-10-29 12:53:40
</commit_message>
<xml_diff>
--- a/02_Areas/工作经历/鑫犇电子有限公司/01_生产部/工程技术组/设备台账.xlsx
+++ b/02_Areas/工作经历/鑫犇电子有限公司/01_生产部/工程技术组/设备台账.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="23">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -149,8 +149,42 @@
       <color rgb="00FF9F0A"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="00171C1D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <i val="1"/>
+      <color rgb="00105186"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00171C1D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="00183A4F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <i val="1"/>
+      <color rgb="00367098"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00183A4F"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -227,8 +261,38 @@
         <fgColor rgb="00FAFAFC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00092B42"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDB338"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00183A4F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0079BBCF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4D7D1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -266,11 +330,31 @@
         <color rgb="000071E3"/>
       </bottom>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D5DDE2"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00092B42"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00B8C6CE"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00183A4F"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -393,6 +477,60 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -867,693 +1005,693 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" s="6">
-      <c r="A1" s="32" t="inlineStr">
+      <c r="A1" s="51" t="inlineStr">
         <is>
           <t>设备编号</t>
         </is>
       </c>
-      <c r="B1" s="32" t="inlineStr">
+      <c r="B1" s="51" t="inlineStr">
         <is>
           <t>设备名称</t>
         </is>
       </c>
-      <c r="C1" s="32" t="inlineStr">
+      <c r="C1" s="51" t="inlineStr">
         <is>
           <t>型号规格</t>
         </is>
       </c>
-      <c r="D1" s="32" t="inlineStr">
+      <c r="D1" s="51" t="inlineStr">
         <is>
           <t>品牌/产地</t>
         </is>
       </c>
-      <c r="E1" s="32" t="inlineStr">
+      <c r="E1" s="51" t="inlineStr">
         <is>
           <t>类别</t>
         </is>
       </c>
-      <c r="F1" s="32" t="inlineStr">
+      <c r="F1" s="51" t="inlineStr">
         <is>
           <t>主要技术参数</t>
         </is>
       </c>
-      <c r="G1" s="32" t="inlineStr">
+      <c r="G1" s="51" t="inlineStr">
         <is>
           <t>工位位置</t>
         </is>
       </c>
-      <c r="H1" s="32" t="inlineStr">
+      <c r="H1" s="51" t="inlineStr">
         <is>
           <t>责任人</t>
         </is>
       </c>
-      <c r="I1" s="32" t="inlineStr">
+      <c r="I1" s="51" t="inlineStr">
         <is>
           <t>当前状态</t>
         </is>
       </c>
-      <c r="J1" s="32" t="inlineStr">
+      <c r="J1" s="51" t="inlineStr">
         <is>
           <t>保养等级</t>
         </is>
       </c>
-      <c r="K1" s="32" t="inlineStr">
+      <c r="K1" s="51" t="inlineStr">
         <is>
           <t>上次保养</t>
         </is>
       </c>
-      <c r="L1" s="32" t="inlineStr">
+      <c r="L1" s="51" t="inlineStr">
         <is>
           <t>下次保养</t>
         </is>
       </c>
-      <c r="M1" s="32" t="inlineStr">
+      <c r="M1" s="51" t="inlineStr">
         <is>
           <t>安全防护</t>
         </is>
       </c>
-      <c r="N1" s="32" t="inlineStr">
+      <c r="N1" s="51" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="O1" s="32" t="inlineStr">
+      <c r="O1" s="51" t="inlineStr">
         <is>
           <t>核对状态</t>
         </is>
       </c>
     </row>
     <row r="2" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A2" s="33" t="inlineStr">
+      <c r="A2" s="52" t="inlineStr">
         <is>
           <t>SB-001</t>
         </is>
       </c>
-      <c r="B2" s="33" t="inlineStr">
+      <c r="B2" s="52" t="inlineStr">
         <is>
           <t>快走丝线切割</t>
         </is>
       </c>
-      <c r="C2" s="33" t="inlineStr">
+      <c r="C2" s="52" t="inlineStr">
         <is>
           <t>DK7732</t>
         </is>
       </c>
-      <c r="D2" s="33" t="inlineStr">
+      <c r="D2" s="52" t="inlineStr">
         <is>
           <t>泰州四海数控</t>
         </is>
       </c>
-      <c r="E2" s="33" t="inlineStr">
+      <c r="E2" s="52" t="inlineStr">
         <is>
           <t>电加工设备</t>
         </is>
       </c>
-      <c r="F2" s="33" t="inlineStr">
+      <c r="F2" s="52" t="inlineStr">
         <is>
           <t>最大加工厚度300mm；锥度±3°；工作台行程320×400mm</t>
         </is>
       </c>
-      <c r="G2" s="33" t="inlineStr">
+      <c r="G2" s="52" t="inlineStr">
         <is>
           <t>模具车间-线切割区</t>
         </is>
       </c>
-      <c r="H2" s="34" t="inlineStr">
+      <c r="H2" s="53" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I2" s="33" t="inlineStr">
+      <c r="I2" s="52" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J2" s="33" t="inlineStr">
+      <c r="J2" s="52" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K2" s="34" t="inlineStr">
+      <c r="K2" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L2" s="34" t="inlineStr">
+      <c r="L2" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M2" s="33" t="inlineStr">
+      <c r="M2" s="52" t="inlineStr">
         <is>
           <t>防护门/急停已配</t>
         </is>
       </c>
-      <c r="N2" s="35" t="inlineStr">
+      <c r="N2" s="54" t="inlineStr">
         <is>
           <t>双机位油槽，带数控系统</t>
         </is>
       </c>
-      <c r="O2" s="34" t="inlineStr">
+      <c r="O2" s="53" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="3" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A3" s="36" t="inlineStr">
+      <c r="A3" s="55" t="inlineStr">
         <is>
           <t>SB-002</t>
         </is>
       </c>
-      <c r="B3" s="36" t="inlineStr">
+      <c r="B3" s="55" t="inlineStr">
         <is>
           <t>锥度线切割</t>
         </is>
       </c>
-      <c r="C3" s="36" t="inlineStr">
+      <c r="C3" s="55" t="inlineStr">
         <is>
           <t>DK7735</t>
         </is>
       </c>
-      <c r="D3" s="36" t="inlineStr">
+      <c r="D3" s="55" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E3" s="36" t="inlineStr">
+      <c r="E3" s="55" t="inlineStr">
         <is>
           <t>电加工设备</t>
         </is>
       </c>
-      <c r="F3" s="36" t="inlineStr">
+      <c r="F3" s="55" t="inlineStr">
         <is>
           <t>最大加工厚度350mm；大锥度切割；工作台行程350×500mm</t>
         </is>
       </c>
-      <c r="G3" s="36" t="inlineStr">
+      <c r="G3" s="55" t="inlineStr">
         <is>
           <t>模具车间-线切割区</t>
         </is>
       </c>
-      <c r="H3" s="37" t="inlineStr">
+      <c r="H3" s="53" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I3" s="36" t="inlineStr">
+      <c r="I3" s="55" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J3" s="36" t="inlineStr">
+      <c r="J3" s="55" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K3" s="37" t="inlineStr">
+      <c r="K3" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L3" s="37" t="inlineStr">
+      <c r="L3" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M3" s="36" t="inlineStr">
+      <c r="M3" s="55" t="inlineStr">
         <is>
           <t>防护门/急停已配</t>
         </is>
       </c>
-      <c r="N3" s="35" t="inlineStr">
+      <c r="N3" s="56" t="inlineStr">
         <is>
           <t>带锥度装置，适合斜度零件</t>
         </is>
       </c>
-      <c r="O3" s="37" t="inlineStr">
+      <c r="O3" s="53" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="4" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A4" s="33" t="inlineStr">
+      <c r="A4" s="52" t="inlineStr">
         <is>
           <t>SB-003</t>
         </is>
       </c>
-      <c r="B4" s="33" t="inlineStr">
+      <c r="B4" s="52" t="inlineStr">
         <is>
           <t>手摇平面磨床</t>
         </is>
       </c>
-      <c r="C4" s="33" t="inlineStr">
+      <c r="C4" s="52" t="inlineStr">
         <is>
           <t>TONVE-618</t>
         </is>
       </c>
-      <c r="D4" s="33" t="inlineStr">
+      <c r="D4" s="52" t="inlineStr">
         <is>
           <t>TONVE通伟</t>
         </is>
       </c>
-      <c r="E4" s="33" t="inlineStr">
+      <c r="E4" s="52" t="inlineStr">
         <is>
           <t>磨削设备</t>
         </is>
       </c>
-      <c r="F4" s="33" t="inlineStr">
+      <c r="F4" s="52" t="inlineStr">
         <is>
           <t>工作台150×450mm；砂轮直径180mm；手动进给</t>
         </is>
       </c>
-      <c r="G4" s="33" t="inlineStr">
+      <c r="G4" s="52" t="inlineStr">
         <is>
           <t>模具车间-磨削区</t>
         </is>
       </c>
-      <c r="H4" s="34" t="inlineStr">
+      <c r="H4" s="53" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I4" s="33" t="inlineStr">
+      <c r="I4" s="52" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J4" s="33" t="inlineStr">
+      <c r="J4" s="52" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K4" s="34" t="inlineStr">
+      <c r="K4" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L4" s="34" t="inlineStr">
+      <c r="L4" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M4" s="33" t="inlineStr">
+      <c r="M4" s="52" t="inlineStr">
         <is>
           <t>砂轮防护罩/吸尘已配</t>
         </is>
       </c>
-      <c r="N4" s="35" t="inlineStr">
+      <c r="N4" s="54" t="inlineStr">
         <is>
           <t>配数显尺，精密小件磨削</t>
         </is>
       </c>
-      <c r="O4" s="34" t="inlineStr">
+      <c r="O4" s="53" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="5" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A5" s="36" t="inlineStr">
+      <c r="A5" s="55" t="inlineStr">
         <is>
           <t>SB-004</t>
         </is>
       </c>
-      <c r="B5" s="36" t="inlineStr">
+      <c r="B5" s="55" t="inlineStr">
         <is>
           <t>台式钻床</t>
         </is>
       </c>
-      <c r="C5" s="36" t="inlineStr">
+      <c r="C5" s="55" t="inlineStr">
         <is>
           <t>WMM-西菱</t>
         </is>
       </c>
-      <c r="D5" s="36" t="inlineStr">
+      <c r="D5" s="55" t="inlineStr">
         <is>
           <t>西菱WMM</t>
         </is>
       </c>
-      <c r="E5" s="36" t="inlineStr">
+      <c r="E5" s="55" t="inlineStr">
         <is>
           <t>钻削设备</t>
         </is>
       </c>
-      <c r="F5" s="36" t="inlineStr">
+      <c r="F5" s="55" t="inlineStr">
         <is>
           <t>最大钻孔直径16mm；工作台圆形；最大行程待补</t>
         </is>
       </c>
-      <c r="G5" s="36" t="inlineStr">
+      <c r="G5" s="55" t="inlineStr">
         <is>
           <t>模具车间-钳工台</t>
         </is>
       </c>
-      <c r="H5" s="37" t="inlineStr">
+      <c r="H5" s="53" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I5" s="36" t="inlineStr">
+      <c r="I5" s="55" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J5" s="36" t="inlineStr">
+      <c r="J5" s="55" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K5" s="37" t="inlineStr">
+      <c r="K5" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L5" s="37" t="inlineStr">
+      <c r="L5" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M5" s="38" t="inlineStr">
+      <c r="M5" s="53" t="inlineStr">
         <is>
           <t>钻夹头钥匙/急停待确认</t>
         </is>
       </c>
-      <c r="N5" s="35" t="inlineStr">
+      <c r="N5" s="56" t="inlineStr">
         <is>
           <t>绿色机身，常规孔加工</t>
         </is>
       </c>
-      <c r="O5" s="37" t="inlineStr">
+      <c r="O5" s="53" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="6" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A6" s="33" t="inlineStr">
+      <c r="A6" s="52" t="inlineStr">
         <is>
           <t>SB-005</t>
         </is>
       </c>
-      <c r="B6" s="33" t="inlineStr">
+      <c r="B6" s="52" t="inlineStr">
         <is>
           <t>立式砂轮机</t>
         </is>
       </c>
-      <c r="C6" s="33" t="inlineStr">
+      <c r="C6" s="52" t="inlineStr">
         <is>
           <t>双工位砂轮机</t>
         </is>
       </c>
-      <c r="D6" s="33" t="inlineStr">
+      <c r="D6" s="52" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E6" s="33" t="inlineStr">
+      <c r="E6" s="52" t="inlineStr">
         <is>
           <t>磨削辅助设备</t>
         </is>
       </c>
-      <c r="F6" s="33" t="inlineStr">
+      <c r="F6" s="52" t="inlineStr">
         <is>
           <t>砂轮直径200mm；双砂轮（白刚玉+绿碳化硅）</t>
         </is>
       </c>
-      <c r="G6" s="33" t="inlineStr">
+      <c r="G6" s="52" t="inlineStr">
         <is>
           <t>模具车间-钳工角</t>
         </is>
       </c>
-      <c r="H6" s="34" t="inlineStr">
+      <c r="H6" s="53" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I6" s="33" t="inlineStr">
+      <c r="I6" s="52" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J6" s="33" t="inlineStr">
+      <c r="J6" s="52" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K6" s="34" t="inlineStr">
+      <c r="K6" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L6" s="34" t="inlineStr">
+      <c r="L6" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M6" s="33" t="inlineStr">
+      <c r="M6" s="52" t="inlineStr">
         <is>
           <t>砂轮防护罩/托架已配</t>
         </is>
       </c>
-      <c r="N6" s="35" t="inlineStr">
+      <c r="N6" s="54" t="inlineStr">
         <is>
           <t>磨刀/去毛刺专用</t>
         </is>
       </c>
-      <c r="O6" s="34" t="inlineStr">
+      <c r="O6" s="53" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="7" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A7" s="36" t="inlineStr">
+      <c r="A7" s="55" t="inlineStr">
         <is>
           <t>SB-006</t>
         </is>
       </c>
-      <c r="B7" s="36" t="inlineStr">
+      <c r="B7" s="55" t="inlineStr">
         <is>
           <t>台式电动冲床</t>
         </is>
       </c>
-      <c r="C7" s="36" t="inlineStr">
+      <c r="C7" s="55" t="inlineStr">
         <is>
           <t>JB04-1T</t>
         </is>
       </c>
-      <c r="D7" s="36" t="inlineStr">
+      <c r="D7" s="55" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E7" s="36" t="inlineStr">
+      <c r="E7" s="55" t="inlineStr">
         <is>
           <t>冲压设备</t>
         </is>
       </c>
-      <c r="F7" s="36" t="inlineStr">
+      <c r="F7" s="55" t="inlineStr">
         <is>
           <t>公称压力1吨；台式；手动按钮操作</t>
         </is>
       </c>
-      <c r="G7" s="36" t="inlineStr">
+      <c r="G7" s="55" t="inlineStr">
         <is>
           <t>模具车间-试模区</t>
         </is>
       </c>
-      <c r="H7" s="37" t="inlineStr">
+      <c r="H7" s="53" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I7" s="36" t="inlineStr">
+      <c r="I7" s="55" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J7" s="36" t="inlineStr">
+      <c r="J7" s="55" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K7" s="37" t="inlineStr">
+      <c r="K7" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L7" s="37" t="inlineStr">
+      <c r="L7" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M7" s="38" t="inlineStr">
+      <c r="M7" s="53" t="inlineStr">
         <is>
           <t>安全光幕/双手按钮待确认</t>
         </is>
       </c>
-      <c r="N7" s="35" t="inlineStr">
+      <c r="N7" s="56" t="inlineStr">
         <is>
           <t>小件试模、冲孔验证</t>
         </is>
       </c>
-      <c r="O7" s="37" t="inlineStr">
+      <c r="O7" s="53" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="8" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A8" s="33" t="inlineStr">
+      <c r="A8" s="52" t="inlineStr">
         <is>
           <t>SB-007</t>
         </is>
       </c>
-      <c r="B8" s="33" t="inlineStr">
+      <c r="B8" s="52" t="inlineStr">
         <is>
           <t>手摇平面磨床</t>
         </is>
       </c>
-      <c r="C8" s="33" t="inlineStr">
+      <c r="C8" s="52" t="inlineStr">
         <is>
           <t>SGM-450</t>
         </is>
       </c>
-      <c r="D8" s="33" t="inlineStr">
+      <c r="D8" s="52" t="inlineStr">
         <is>
           <t>曙光SHUGUANG</t>
         </is>
       </c>
-      <c r="E8" s="33" t="inlineStr">
+      <c r="E8" s="52" t="inlineStr">
         <is>
           <t>磨削设备</t>
         </is>
       </c>
-      <c r="F8" s="33" t="inlineStr">
+      <c r="F8" s="52" t="inlineStr">
         <is>
           <t>工作台150×450mm；砂轮直径200mm；数显尺寸</t>
         </is>
       </c>
-      <c r="G8" s="33" t="inlineStr">
+      <c r="G8" s="52" t="inlineStr">
         <is>
           <t>模具车间-磨削区</t>
         </is>
       </c>
-      <c r="H8" s="34" t="inlineStr">
+      <c r="H8" s="53" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I8" s="33" t="inlineStr">
+      <c r="I8" s="52" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J8" s="33" t="inlineStr">
+      <c r="J8" s="52" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K8" s="34" t="inlineStr">
+      <c r="K8" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L8" s="34" t="inlineStr">
+      <c r="L8" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M8" s="33" t="inlineStr">
+      <c r="M8" s="52" t="inlineStr">
         <is>
           <t>砂轮防护罩/吸尘已配</t>
         </is>
       </c>
-      <c r="N8" s="35" t="inlineStr">
+      <c r="N8" s="54" t="inlineStr">
         <is>
           <t>与TONVE并排，配数显</t>
         </is>
       </c>
-      <c r="O8" s="34" t="inlineStr">
+      <c r="O8" s="53" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
     <row r="9" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A9" s="36" t="inlineStr">
+      <c r="A9" s="55" t="inlineStr">
         <is>
           <t>SB-008</t>
         </is>
       </c>
-      <c r="B9" s="36" t="inlineStr">
+      <c r="B9" s="55" t="inlineStr">
         <is>
           <t>台式仪表车床</t>
         </is>
       </c>
-      <c r="C9" s="36" t="inlineStr">
+      <c r="C9" s="55" t="inlineStr">
         <is>
           <t>CJ0625B</t>
         </is>
       </c>
-      <c r="D9" s="36" t="inlineStr">
+      <c r="D9" s="55" t="inlineStr">
         <is>
           <t>恒生机床</t>
         </is>
       </c>
-      <c r="E9" s="36" t="inlineStr">
+      <c r="E9" s="55" t="inlineStr">
         <is>
           <t>车削设备</t>
         </is>
       </c>
-      <c r="F9" s="36" t="inlineStr">
+      <c r="F9" s="55" t="inlineStr">
         <is>
           <t>最大回转直径250mm；最大加工长度300mm；手动进给</t>
         </is>
       </c>
-      <c r="G9" s="36" t="inlineStr">
+      <c r="G9" s="55" t="inlineStr">
         <is>
           <t>模具车间-钳工台旁</t>
         </is>
       </c>
-      <c r="H9" s="37" t="inlineStr">
+      <c r="H9" s="53" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I9" s="36" t="inlineStr">
+      <c r="I9" s="55" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J9" s="36" t="inlineStr">
+      <c r="J9" s="55" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K9" s="37" t="inlineStr">
+      <c r="K9" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L9" s="37" t="inlineStr">
+      <c r="L9" s="53" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M9" s="38" t="inlineStr">
+      <c r="M9" s="53" t="inlineStr">
         <is>
           <t>卡盘扳手/防护待确认</t>
         </is>
       </c>
-      <c r="N9" s="35" t="inlineStr">
+      <c r="N9" s="56" t="inlineStr">
         <is>
           <t>小件车削、螺纹加工</t>
         </is>
       </c>
-      <c r="O9" s="37" t="inlineStr">
+      <c r="O9" s="53" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
@@ -1594,114 +1732,114 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="57" t="inlineStr">
         <is>
           <t>设备台账使用说明</t>
         </is>
       </c>
-      <c r="B1" s="39" t="n"/>
+      <c r="B1" s="57" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="40" t="n"/>
-      <c r="B2" s="40" t="n"/>
+      <c r="A2" s="58" t="n"/>
+      <c r="B2" s="58" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="40" t="inlineStr">
+      <c r="A3" s="58" t="inlineStr">
         <is>
           <t>1. 设备编号规则</t>
         </is>
       </c>
-      <c r="B3" s="40" t="inlineStr">
+      <c r="B3" s="58" t="inlineStr">
         <is>
           <t>SB-序号，按车间统一编号，一台一码，终身不变</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="40" t="inlineStr">
+      <c r="A4" s="58" t="inlineStr">
         <is>
           <t>2. 责任人</t>
         </is>
       </c>
-      <c r="B4" s="40" t="inlineStr">
+      <c r="B4" s="58" t="inlineStr">
         <is>
           <t>由生产主管指定，每台设备定岗到人</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="40" t="inlineStr">
+      <c r="A5" s="58" t="inlineStr">
         <is>
           <t>3. 当前状态</t>
         </is>
       </c>
-      <c r="B5" s="40" t="inlineStr">
+      <c r="B5" s="58" t="inlineStr">
         <is>
           <t>在用 / 待修 / 封存 / 报废</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="40" t="inlineStr">
+      <c r="A6" s="58" t="inlineStr">
         <is>
           <t>4. 保养等级</t>
         </is>
       </c>
-      <c r="B6" s="40" t="inlineStr">
+      <c r="B6" s="58" t="inlineStr">
         <is>
           <t>日点检（操作工）/ 周保养（班组长）/ 月保养（设备管理员）/ 年保养（外部）</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="40" t="inlineStr">
+      <c r="A7" s="58" t="inlineStr">
         <is>
           <t>5. 安全防护</t>
         </is>
       </c>
-      <c r="B7" s="40" t="inlineStr">
+      <c r="B7" s="58" t="inlineStr">
         <is>
           <t>开机前必须确认防护装置齐全有效</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="40" t="inlineStr">
+      <c r="A8" s="58" t="inlineStr">
         <is>
           <t>6. 备注</t>
         </is>
       </c>
-      <c r="B8" s="40" t="inlineStr">
+      <c r="B8" s="58" t="inlineStr">
         <is>
           <t>记录设备特殊用途、夹具、常用加工零件型号等</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="40" t="n"/>
-      <c r="B9" s="40" t="n"/>
+      <c r="A9" s="58" t="n"/>
+      <c r="B9" s="58" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="40" t="inlineStr">
+      <c r="A10" s="58" t="inlineStr">
         <is>
           <t>更新说明</t>
         </is>
       </c>
-      <c r="B10" s="40" t="inlineStr">
+      <c r="B10" s="58" t="inlineStr">
         <is>
           <t>本次为知识库设备台账更新优化：保留原有8条设备记录，增加筛选、表格化、下拉选项和核对状态；不将照片或现有文字当作最终铭牌/安全验收结论。</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="41" t="inlineStr">
-        <is>
-          <t>配色规范</t>
-        </is>
-      </c>
-      <c r="B11" s="35" t="inlineStr">
-        <is>
-          <t>苹果式浅色界面取向：白色/极浅灰为主，深灰为正文，系统蓝仅作结构强调，红色仅表示待确认/待补，橙色仅表示安全关注；不使用大面积深色底、不使用同色底字。</t>
+      <c r="A11" s="59" t="inlineStr">
+        <is>
+          <t>定版配色</t>
+        </is>
+      </c>
+      <c r="B11" s="56" t="inlineStr">
+        <is>
+          <t>本工作簿统一使用蓝灰配色：#2C5B82、#367098、#D4D7D1、#79BBCF、#183A4F。除白字表头外，不引入红、黄、橙、绿等其他强调色。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-10-29 13:04:37
</commit_message>
<xml_diff>
--- a/02_Areas/工作经历/鑫犇电子有限公司/01_生产部/工程技术组/设备台账.xlsx
+++ b/02_Areas/工作经历/鑫犇电子有限公司/01_生产部/工程技术组/设备台账.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'设备台账'!$A$1:$O$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'设备台账'!$A$4:$O$12</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="29">
+  <fonts count="33">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -182,6 +182,30 @@
       <b val="1"/>
       <color rgb="00183A4F"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00367098"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00183A4F"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <i val="1"/>
+      <color rgb="00367098"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="22">
@@ -354,7 +378,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -532,6 +556,48 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="21" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="21" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -615,21 +681,6 @@
     <author>Hermes</author>
   </authors>
   <commentList>
-    <comment ref="O2" authorId="0" shapeId="0">
-      <text>
-        <t>核对状态仅表示台账资料与现场铭牌/设备状态的核对进度，不等同于安全验收合格。</t>
-      </text>
-    </comment>
-    <comment ref="O3" authorId="0" shapeId="0">
-      <text>
-        <t>核对状态仅表示台账资料与现场铭牌/设备状态的核对进度，不等同于安全验收合格。</t>
-      </text>
-    </comment>
-    <comment ref="O4" authorId="0" shapeId="0">
-      <text>
-        <t>核对状态仅表示台账资料与现场铭牌/设备状态的核对进度，不等同于安全验收合格。</t>
-      </text>
-    </comment>
     <comment ref="O5" authorId="0" shapeId="0">
       <text>
         <t>核对状态仅表示台账资料与现场铭牌/设备状态的核对进度，不等同于安全验收合格。</t>
@@ -655,13 +706,28 @@
         <t>核对状态仅表示台账资料与现场铭牌/设备状态的核对进度，不等同于安全验收合格。</t>
       </text>
     </comment>
+    <comment ref="O10" authorId="0" shapeId="0">
+      <text>
+        <t>核对状态仅表示台账资料与现场铭牌/设备状态的核对进度，不等同于安全验收合格。</t>
+      </text>
+    </comment>
+    <comment ref="O11" authorId="0" shapeId="0">
+      <text>
+        <t>核对状态仅表示台账资料与现场铭牌/设备状态的核对进度，不等同于安全验收合格。</t>
+      </text>
+    </comment>
+    <comment ref="O12" authorId="0" shapeId="0">
+      <text>
+        <t>核对状态仅表示台账资料与现场铭牌/设备状态的核对进度，不等同于安全验收合格。</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EquipmentRegister" displayName="EquipmentRegister" ref="A1:O9" headerRowCount="1">
-  <autoFilter ref="A1:O9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EquipmentRegister" displayName="EquipmentRegister" ref="A4:O12" headerRowCount="1">
+  <autoFilter ref="A4:O12"/>
   <tableColumns count="15">
     <tableColumn id="1" name="设备编号"/>
     <tableColumn id="2" name="设备名称"/>
@@ -984,721 +1050,784 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.466666666666667" defaultRowHeight="18.66666666666666"/>
   <cols>
     <col width="12" customWidth="1" style="6" min="1" max="1"/>
     <col width="18" customWidth="1" style="6" min="2" max="2"/>
-    <col width="16" customWidth="1" style="6" min="3" max="3"/>
-    <col width="18" customWidth="1" style="6" min="4" max="4"/>
-    <col width="16" customWidth="1" style="6" min="5" max="5"/>
-    <col width="44" customWidth="1" style="6" min="6" max="6"/>
-    <col width="24" customWidth="1" style="6" min="7" max="7"/>
+    <col width="15" customWidth="1" style="6" min="3" max="3"/>
+    <col width="17" customWidth="1" style="6" min="4" max="4"/>
+    <col width="15" customWidth="1" style="6" min="5" max="5"/>
+    <col width="38" customWidth="1" style="6" min="6" max="6"/>
+    <col width="22" customWidth="1" style="6" min="7" max="7"/>
     <col width="12" customWidth="1" style="6" min="8" max="8"/>
     <col width="12" customWidth="1" style="6" min="9" max="9"/>
     <col width="12" customWidth="1" style="6" min="10" max="10"/>
     <col width="12" customWidth="1" style="6" min="11" max="11"/>
     <col width="12" customWidth="1" style="6" min="12" max="12"/>
-    <col width="24" customWidth="1" style="6" min="13" max="13"/>
-    <col width="32" customWidth="1" style="6" min="14" max="14"/>
+    <col width="25" customWidth="1" style="6" min="13" max="13"/>
+    <col width="30" customWidth="1" style="6" min="14" max="14"/>
     <col width="16" customWidth="1" style="6" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" s="6">
-      <c r="A1" s="51" t="inlineStr">
+    <row r="1" ht="30" customHeight="1" s="6">
+      <c r="A1" s="60" t="inlineStr">
+        <is>
+          <t>工程技术组｜设备台账</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1" s="6">
+      <c r="A2" s="61" t="inlineStr">
+        <is>
+          <t>设备总数</t>
+        </is>
+      </c>
+      <c r="B2" s="62">
+        <f>COUNTA(A5:A12)</f>
+        <v/>
+      </c>
+      <c r="C2" s="63" t="n"/>
+      <c r="D2" s="61" t="inlineStr">
+        <is>
+          <t>当前登记在用</t>
+        </is>
+      </c>
+      <c r="E2" s="62">
+        <f>COUNTIF(I5:I12,"在用")</f>
+        <v/>
+      </c>
+      <c r="F2" s="63" t="n"/>
+      <c r="G2" s="61" t="inlineStr">
+        <is>
+          <t>责任人待指定</t>
+        </is>
+      </c>
+      <c r="H2" s="62">
+        <f>COUNTIF(H5:H12,"待指定")</f>
+        <v/>
+      </c>
+      <c r="I2" s="63" t="n"/>
+      <c r="J2" s="61" t="inlineStr">
+        <is>
+          <t>现场核对待完成</t>
+        </is>
+      </c>
+      <c r="K2" s="62">
+        <f>COUNTIF(O5:O12,"待现场核对")</f>
+        <v/>
+      </c>
+      <c r="L2" s="63" t="n"/>
+      <c r="M2" s="63" t="n"/>
+      <c r="N2" s="63" t="n"/>
+      <c r="O2" s="63" t="n"/>
+    </row>
+    <row r="3" ht="24" customHeight="1" s="6">
+      <c r="A3" s="64" t="inlineStr">
+        <is>
+          <t>说明：台账数据保留现状记录；“在用”仅表示当前登记状态，铭牌、责任人、安全防护和现场核对仍以实际确认结果为准。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1" s="6">
+      <c r="A4" s="51" t="inlineStr">
         <is>
           <t>设备编号</t>
         </is>
       </c>
-      <c r="B1" s="51" t="inlineStr">
+      <c r="B4" s="51" t="inlineStr">
         <is>
           <t>设备名称</t>
         </is>
       </c>
-      <c r="C1" s="51" t="inlineStr">
+      <c r="C4" s="51" t="inlineStr">
         <is>
           <t>型号规格</t>
         </is>
       </c>
-      <c r="D1" s="51" t="inlineStr">
+      <c r="D4" s="51" t="inlineStr">
         <is>
           <t>品牌/产地</t>
         </is>
       </c>
-      <c r="E1" s="51" t="inlineStr">
+      <c r="E4" s="51" t="inlineStr">
         <is>
           <t>类别</t>
         </is>
       </c>
-      <c r="F1" s="51" t="inlineStr">
+      <c r="F4" s="51" t="inlineStr">
         <is>
           <t>主要技术参数</t>
         </is>
       </c>
-      <c r="G1" s="51" t="inlineStr">
+      <c r="G4" s="51" t="inlineStr">
         <is>
           <t>工位位置</t>
         </is>
       </c>
-      <c r="H1" s="51" t="inlineStr">
+      <c r="H4" s="51" t="inlineStr">
         <is>
           <t>责任人</t>
         </is>
       </c>
-      <c r="I1" s="51" t="inlineStr">
+      <c r="I4" s="51" t="inlineStr">
         <is>
           <t>当前状态</t>
         </is>
       </c>
-      <c r="J1" s="51" t="inlineStr">
+      <c r="J4" s="51" t="inlineStr">
         <is>
           <t>保养等级</t>
         </is>
       </c>
-      <c r="K1" s="51" t="inlineStr">
+      <c r="K4" s="51" t="inlineStr">
         <is>
           <t>上次保养</t>
         </is>
       </c>
-      <c r="L1" s="51" t="inlineStr">
+      <c r="L4" s="51" t="inlineStr">
         <is>
           <t>下次保养</t>
         </is>
       </c>
-      <c r="M1" s="51" t="inlineStr">
+      <c r="M4" s="51" t="inlineStr">
         <is>
           <t>安全防护</t>
         </is>
       </c>
-      <c r="N1" s="51" t="inlineStr">
+      <c r="N4" s="51" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="O1" s="51" t="inlineStr">
+      <c r="O4" s="51" t="inlineStr">
         <is>
           <t>核对状态</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A2" s="52" t="inlineStr">
+    <row r="5" ht="49.77777777777778" customHeight="1" s="6">
+      <c r="A5" s="65" t="inlineStr">
         <is>
           <t>SB-001</t>
         </is>
       </c>
-      <c r="B2" s="52" t="inlineStr">
+      <c r="B5" s="66" t="inlineStr">
         <is>
           <t>快走丝线切割</t>
         </is>
       </c>
-      <c r="C2" s="52" t="inlineStr">
+      <c r="C5" s="65" t="inlineStr">
         <is>
           <t>DK7732</t>
         </is>
       </c>
-      <c r="D2" s="52" t="inlineStr">
+      <c r="D5" s="66" t="inlineStr">
         <is>
           <t>泰州四海数控</t>
         </is>
       </c>
-      <c r="E2" s="52" t="inlineStr">
+      <c r="E5" s="65" t="inlineStr">
         <is>
           <t>电加工设备</t>
         </is>
       </c>
-      <c r="F2" s="52" t="inlineStr">
+      <c r="F5" s="66" t="inlineStr">
         <is>
           <t>最大加工厚度300mm；锥度±3°；工作台行程320×400mm</t>
         </is>
       </c>
-      <c r="G2" s="52" t="inlineStr">
+      <c r="G5" s="66" t="inlineStr">
         <is>
           <t>模具车间-线切割区</t>
         </is>
       </c>
-      <c r="H2" s="53" t="inlineStr">
+      <c r="H5" s="67" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I2" s="52" t="inlineStr">
+      <c r="I5" s="68" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J2" s="52" t="inlineStr">
+      <c r="J5" s="65" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K2" s="53" t="inlineStr">
+      <c r="K5" s="67" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L2" s="53" t="inlineStr">
+      <c r="L5" s="69" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M2" s="52" t="inlineStr">
+      <c r="M5" s="66" t="inlineStr">
         <is>
           <t>防护门/急停已配</t>
         </is>
       </c>
-      <c r="N2" s="54" t="inlineStr">
+      <c r="N5" s="70" t="inlineStr">
         <is>
           <t>双机位油槽，带数控系统</t>
         </is>
       </c>
-      <c r="O2" s="53" t="inlineStr">
+      <c r="O5" s="67" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A3" s="55" t="inlineStr">
+    <row r="6" ht="49.77777777777778" customHeight="1" s="6">
+      <c r="A6" s="71" t="inlineStr">
         <is>
           <t>SB-002</t>
         </is>
       </c>
-      <c r="B3" s="55" t="inlineStr">
+      <c r="B6" s="72" t="inlineStr">
         <is>
           <t>锥度线切割</t>
         </is>
       </c>
-      <c r="C3" s="55" t="inlineStr">
+      <c r="C6" s="71" t="inlineStr">
         <is>
           <t>DK7735</t>
         </is>
       </c>
-      <c r="D3" s="55" t="inlineStr">
+      <c r="D6" s="72" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E3" s="55" t="inlineStr">
+      <c r="E6" s="71" t="inlineStr">
         <is>
           <t>电加工设备</t>
         </is>
       </c>
-      <c r="F3" s="55" t="inlineStr">
+      <c r="F6" s="72" t="inlineStr">
         <is>
           <t>最大加工厚度350mm；大锥度切割；工作台行程350×500mm</t>
         </is>
       </c>
-      <c r="G3" s="55" t="inlineStr">
+      <c r="G6" s="72" t="inlineStr">
         <is>
           <t>模具车间-线切割区</t>
         </is>
       </c>
-      <c r="H3" s="53" t="inlineStr">
+      <c r="H6" s="67" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I3" s="55" t="inlineStr">
+      <c r="I6" s="68" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J3" s="55" t="inlineStr">
+      <c r="J6" s="71" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K3" s="53" t="inlineStr">
+      <c r="K6" s="67" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L3" s="53" t="inlineStr">
+      <c r="L6" s="69" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M3" s="55" t="inlineStr">
+      <c r="M6" s="72" t="inlineStr">
         <is>
           <t>防护门/急停已配</t>
         </is>
       </c>
-      <c r="N3" s="56" t="inlineStr">
+      <c r="N6" s="73" t="inlineStr">
         <is>
           <t>带锥度装置，适合斜度零件</t>
         </is>
       </c>
-      <c r="O3" s="53" t="inlineStr">
+      <c r="O6" s="67" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A4" s="52" t="inlineStr">
+    <row r="7" ht="49.77777777777778" customHeight="1" s="6">
+      <c r="A7" s="65" t="inlineStr">
         <is>
           <t>SB-003</t>
         </is>
       </c>
-      <c r="B4" s="52" t="inlineStr">
+      <c r="B7" s="66" t="inlineStr">
         <is>
           <t>手摇平面磨床</t>
         </is>
       </c>
-      <c r="C4" s="52" t="inlineStr">
+      <c r="C7" s="65" t="inlineStr">
         <is>
           <t>TONVE-618</t>
         </is>
       </c>
-      <c r="D4" s="52" t="inlineStr">
+      <c r="D7" s="66" t="inlineStr">
         <is>
           <t>TONVE通伟</t>
         </is>
       </c>
-      <c r="E4" s="52" t="inlineStr">
+      <c r="E7" s="65" t="inlineStr">
         <is>
           <t>磨削设备</t>
         </is>
       </c>
-      <c r="F4" s="52" t="inlineStr">
+      <c r="F7" s="66" t="inlineStr">
         <is>
           <t>工作台150×450mm；砂轮直径180mm；手动进给</t>
         </is>
       </c>
-      <c r="G4" s="52" t="inlineStr">
+      <c r="G7" s="66" t="inlineStr">
         <is>
           <t>模具车间-磨削区</t>
         </is>
       </c>
-      <c r="H4" s="53" t="inlineStr">
+      <c r="H7" s="67" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I4" s="52" t="inlineStr">
+      <c r="I7" s="68" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J4" s="52" t="inlineStr">
+      <c r="J7" s="65" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K4" s="53" t="inlineStr">
+      <c r="K7" s="67" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L4" s="53" t="inlineStr">
+      <c r="L7" s="69" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M4" s="52" t="inlineStr">
+      <c r="M7" s="66" t="inlineStr">
         <is>
           <t>砂轮防护罩/吸尘已配</t>
         </is>
       </c>
-      <c r="N4" s="54" t="inlineStr">
+      <c r="N7" s="70" t="inlineStr">
         <is>
           <t>配数显尺，精密小件磨削</t>
         </is>
       </c>
-      <c r="O4" s="53" t="inlineStr">
+      <c r="O7" s="67" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A5" s="55" t="inlineStr">
+    <row r="8" ht="49.77777777777778" customHeight="1" s="6">
+      <c r="A8" s="71" t="inlineStr">
         <is>
           <t>SB-004</t>
         </is>
       </c>
-      <c r="B5" s="55" t="inlineStr">
+      <c r="B8" s="72" t="inlineStr">
         <is>
           <t>台式钻床</t>
         </is>
       </c>
-      <c r="C5" s="55" t="inlineStr">
+      <c r="C8" s="71" t="inlineStr">
         <is>
           <t>WMM-西菱</t>
         </is>
       </c>
-      <c r="D5" s="55" t="inlineStr">
+      <c r="D8" s="72" t="inlineStr">
         <is>
           <t>西菱WMM</t>
         </is>
       </c>
-      <c r="E5" s="55" t="inlineStr">
+      <c r="E8" s="71" t="inlineStr">
         <is>
           <t>钻削设备</t>
         </is>
       </c>
-      <c r="F5" s="55" t="inlineStr">
+      <c r="F8" s="72" t="inlineStr">
         <is>
           <t>最大钻孔直径16mm；工作台圆形；最大行程待补</t>
         </is>
       </c>
-      <c r="G5" s="55" t="inlineStr">
+      <c r="G8" s="72" t="inlineStr">
         <is>
           <t>模具车间-钳工台</t>
         </is>
       </c>
-      <c r="H5" s="53" t="inlineStr">
+      <c r="H8" s="67" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I5" s="55" t="inlineStr">
+      <c r="I8" s="68" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J5" s="55" t="inlineStr">
+      <c r="J8" s="71" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K5" s="53" t="inlineStr">
+      <c r="K8" s="67" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L5" s="53" t="inlineStr">
+      <c r="L8" s="69" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M5" s="53" t="inlineStr">
+      <c r="M8" s="72" t="inlineStr">
         <is>
           <t>钻夹头钥匙/急停待确认</t>
         </is>
       </c>
-      <c r="N5" s="56" t="inlineStr">
+      <c r="N8" s="73" t="inlineStr">
         <is>
           <t>绿色机身，常规孔加工</t>
         </is>
       </c>
-      <c r="O5" s="53" t="inlineStr">
+      <c r="O8" s="67" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A6" s="52" t="inlineStr">
+    <row r="9" ht="49.77777777777778" customHeight="1" s="6">
+      <c r="A9" s="65" t="inlineStr">
         <is>
           <t>SB-005</t>
         </is>
       </c>
-      <c r="B6" s="52" t="inlineStr">
+      <c r="B9" s="66" t="inlineStr">
         <is>
           <t>立式砂轮机</t>
         </is>
       </c>
-      <c r="C6" s="52" t="inlineStr">
+      <c r="C9" s="65" t="inlineStr">
         <is>
           <t>双工位砂轮机</t>
         </is>
       </c>
-      <c r="D6" s="52" t="inlineStr">
+      <c r="D9" s="66" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E6" s="52" t="inlineStr">
+      <c r="E9" s="65" t="inlineStr">
         <is>
           <t>磨削辅助设备</t>
         </is>
       </c>
-      <c r="F6" s="52" t="inlineStr">
+      <c r="F9" s="66" t="inlineStr">
         <is>
           <t>砂轮直径200mm；双砂轮（白刚玉+绿碳化硅）</t>
         </is>
       </c>
-      <c r="G6" s="52" t="inlineStr">
+      <c r="G9" s="66" t="inlineStr">
         <is>
           <t>模具车间-钳工角</t>
         </is>
       </c>
-      <c r="H6" s="53" t="inlineStr">
+      <c r="H9" s="67" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I6" s="52" t="inlineStr">
+      <c r="I9" s="68" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J6" s="52" t="inlineStr">
+      <c r="J9" s="65" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K6" s="53" t="inlineStr">
+      <c r="K9" s="67" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L6" s="53" t="inlineStr">
+      <c r="L9" s="69" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M6" s="52" t="inlineStr">
+      <c r="M9" s="66" t="inlineStr">
         <is>
           <t>砂轮防护罩/托架已配</t>
         </is>
       </c>
-      <c r="N6" s="54" t="inlineStr">
+      <c r="N9" s="70" t="inlineStr">
         <is>
           <t>磨刀/去毛刺专用</t>
         </is>
       </c>
-      <c r="O6" s="53" t="inlineStr">
+      <c r="O9" s="67" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A7" s="55" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="71" t="inlineStr">
         <is>
           <t>SB-006</t>
         </is>
       </c>
-      <c r="B7" s="55" t="inlineStr">
+      <c r="B10" s="72" t="inlineStr">
         <is>
           <t>台式电动冲床</t>
         </is>
       </c>
-      <c r="C7" s="55" t="inlineStr">
+      <c r="C10" s="71" t="inlineStr">
         <is>
           <t>JB04-1T</t>
         </is>
       </c>
-      <c r="D7" s="55" t="inlineStr">
+      <c r="D10" s="72" t="inlineStr">
         <is>
           <t>国产</t>
         </is>
       </c>
-      <c r="E7" s="55" t="inlineStr">
+      <c r="E10" s="71" t="inlineStr">
         <is>
           <t>冲压设备</t>
         </is>
       </c>
-      <c r="F7" s="55" t="inlineStr">
+      <c r="F10" s="72" t="inlineStr">
         <is>
           <t>公称压力1吨；台式；手动按钮操作</t>
         </is>
       </c>
-      <c r="G7" s="55" t="inlineStr">
+      <c r="G10" s="72" t="inlineStr">
         <is>
           <t>模具车间-试模区</t>
         </is>
       </c>
-      <c r="H7" s="53" t="inlineStr">
+      <c r="H10" s="67" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I7" s="55" t="inlineStr">
+      <c r="I10" s="68" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J7" s="55" t="inlineStr">
+      <c r="J10" s="71" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K7" s="53" t="inlineStr">
+      <c r="K10" s="67" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L7" s="53" t="inlineStr">
+      <c r="L10" s="69" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M7" s="53" t="inlineStr">
+      <c r="M10" s="72" t="inlineStr">
         <is>
           <t>安全光幕/双手按钮待确认</t>
         </is>
       </c>
-      <c r="N7" s="56" t="inlineStr">
+      <c r="N10" s="73" t="inlineStr">
         <is>
           <t>小件试模、冲孔验证</t>
         </is>
       </c>
-      <c r="O7" s="53" t="inlineStr">
+      <c r="O10" s="67" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A8" s="52" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="65" t="inlineStr">
         <is>
           <t>SB-007</t>
         </is>
       </c>
-      <c r="B8" s="52" t="inlineStr">
+      <c r="B11" s="66" t="inlineStr">
         <is>
           <t>手摇平面磨床</t>
         </is>
       </c>
-      <c r="C8" s="52" t="inlineStr">
+      <c r="C11" s="65" t="inlineStr">
         <is>
           <t>SGM-450</t>
         </is>
       </c>
-      <c r="D8" s="52" t="inlineStr">
+      <c r="D11" s="66" t="inlineStr">
         <is>
           <t>曙光SHUGUANG</t>
         </is>
       </c>
-      <c r="E8" s="52" t="inlineStr">
+      <c r="E11" s="65" t="inlineStr">
         <is>
           <t>磨削设备</t>
         </is>
       </c>
-      <c r="F8" s="52" t="inlineStr">
+      <c r="F11" s="66" t="inlineStr">
         <is>
           <t>工作台150×450mm；砂轮直径200mm；数显尺寸</t>
         </is>
       </c>
-      <c r="G8" s="52" t="inlineStr">
+      <c r="G11" s="66" t="inlineStr">
         <is>
           <t>模具车间-磨削区</t>
         </is>
       </c>
-      <c r="H8" s="53" t="inlineStr">
+      <c r="H11" s="67" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I8" s="52" t="inlineStr">
+      <c r="I11" s="68" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J8" s="52" t="inlineStr">
+      <c r="J11" s="65" t="inlineStr">
         <is>
           <t>周度保养</t>
         </is>
       </c>
-      <c r="K8" s="53" t="inlineStr">
+      <c r="K11" s="67" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L8" s="53" t="inlineStr">
+      <c r="L11" s="69" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M8" s="52" t="inlineStr">
+      <c r="M11" s="66" t="inlineStr">
         <is>
           <t>砂轮防护罩/吸尘已配</t>
         </is>
       </c>
-      <c r="N8" s="54" t="inlineStr">
+      <c r="N11" s="70" t="inlineStr">
         <is>
           <t>与TONVE并排，配数显</t>
         </is>
       </c>
-      <c r="O8" s="53" t="inlineStr">
+      <c r="O11" s="67" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="49.77777777777778" customHeight="1" s="6">
-      <c r="A9" s="55" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="71" t="inlineStr">
         <is>
           <t>SB-008</t>
         </is>
       </c>
-      <c r="B9" s="55" t="inlineStr">
+      <c r="B12" s="72" t="inlineStr">
         <is>
           <t>台式仪表车床</t>
         </is>
       </c>
-      <c r="C9" s="55" t="inlineStr">
+      <c r="C12" s="71" t="inlineStr">
         <is>
           <t>CJ0625B</t>
         </is>
       </c>
-      <c r="D9" s="55" t="inlineStr">
+      <c r="D12" s="72" t="inlineStr">
         <is>
           <t>恒生机床</t>
         </is>
       </c>
-      <c r="E9" s="55" t="inlineStr">
+      <c r="E12" s="71" t="inlineStr">
         <is>
           <t>车削设备</t>
         </is>
       </c>
-      <c r="F9" s="55" t="inlineStr">
+      <c r="F12" s="72" t="inlineStr">
         <is>
           <t>最大回转直径250mm；最大加工长度300mm；手动进给</t>
         </is>
       </c>
-      <c r="G9" s="55" t="inlineStr">
+      <c r="G12" s="72" t="inlineStr">
         <is>
           <t>模具车间-钳工台旁</t>
         </is>
       </c>
-      <c r="H9" s="53" t="inlineStr">
+      <c r="H12" s="67" t="inlineStr">
         <is>
           <t>待指定</t>
         </is>
       </c>
-      <c r="I9" s="55" t="inlineStr">
+      <c r="I12" s="68" t="inlineStr">
         <is>
           <t>在用</t>
         </is>
       </c>
-      <c r="J9" s="55" t="inlineStr">
+      <c r="J12" s="71" t="inlineStr">
         <is>
           <t>月度保养</t>
         </is>
       </c>
-      <c r="K9" s="53" t="inlineStr">
+      <c r="K12" s="67" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="L9" s="53" t="inlineStr">
+      <c r="L12" s="69" t="inlineStr">
         <is>
           <t>待补</t>
         </is>
       </c>
-      <c r="M9" s="53" t="inlineStr">
+      <c r="M12" s="72" t="inlineStr">
         <is>
           <t>卡盘扳手/防护待确认</t>
         </is>
       </c>
-      <c r="N9" s="56" t="inlineStr">
+      <c r="N12" s="73" t="inlineStr">
         <is>
           <t>小件车削、螺纹加工</t>
         </is>
       </c>
-      <c r="O9" s="53" t="inlineStr">
+      <c r="O12" s="67" t="inlineStr">
         <is>
           <t>待现场核对</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O9"/>
+  <autoFilter ref="A4:O12"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A3:O3"/>
+  </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="I2:I9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"在用,停用,维修,报废,待确认"</formula1>
@@ -1834,12 +1963,12 @@
     <row r="11">
       <c r="A11" s="59" t="inlineStr">
         <is>
-          <t>定版配色</t>
+          <t>布局优化说明</t>
         </is>
       </c>
       <c r="B11" s="56" t="inlineStr">
         <is>
-          <t>本工作簿统一使用蓝灰配色：#2C5B82、#367098、#D4D7D1、#79BBCF、#183A4F。除白字表头外，不引入红、黄、橙、绿等其他强调色。</t>
+          <t>本次按国际管理表格设计语言优化：标题与摘要先行；表头、数据区、状态标签分层；减少竖向网格；冻结首列和表头；按阅读动线安排字段；保留统一蓝灰配色，不引入其他颜色。</t>
         </is>
       </c>
     </row>

</xml_diff>